<commit_message>
update rka dari web
</commit_message>
<xml_diff>
--- a/data/rka.xlsx
+++ b/data/rka.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x15 xr xr6 xr10">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
@@ -8,15 +8,25 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\3. TSSP.3\1. Laporan Bulanan\2026\3. Mar\KP\RKA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:40009_{5E5466EE-E6E1-429B-BCEC-F0A77692F222}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D7A97A4-4776-4D35-86D1-586F803A99F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Budget 3 Juni 2024" sheetId="1" r:id="rId1"/>
+    <sheet name="II PD" sheetId="3" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
   <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
       <xlwcv:version setVersion="1"/>
     </ext>
@@ -25,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="554" uniqueCount="151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="616" uniqueCount="152">
   <si>
     <t>Funds Center/Commitment Item</t>
   </si>
@@ -479,11 +489,18 @@
   <si>
     <t>32020100 Prasarana</t>
   </si>
+  <si>
+    <t>RKAO Disetujui</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="2">
+    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="164" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
+  </numFmts>
   <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -620,7 +637,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="34">
+  <fills count="35">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -806,6 +823,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="10">
     <border>
@@ -923,7 +946,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="42">
+  <cellStyleXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
@@ -966,14 +989,33 @@
     <xf numFmtId="0" fontId="1" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="42" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="34" borderId="0" xfId="42" applyNumberFormat="1" applyFont="1" applyFill="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="42" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="34" borderId="0" xfId="42" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="42" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="34" borderId="0" xfId="42" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="42" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="42" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="42">
+  <cellStyles count="43">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
     <cellStyle name="20% - Accent2" xfId="23" builtinId="34" customBuiltin="1"/>
     <cellStyle name="20% - Accent3" xfId="27" builtinId="38" customBuiltin="1"/>
@@ -1001,6 +1043,7 @@
     <cellStyle name="Bad" xfId="7" builtinId="27" customBuiltin="1"/>
     <cellStyle name="Calculation" xfId="11" builtinId="22" customBuiltin="1"/>
     <cellStyle name="Check Cell" xfId="13" builtinId="23" customBuiltin="1"/>
+    <cellStyle name="Comma" xfId="42" builtinId="3"/>
     <cellStyle name="Explanatory Text" xfId="16" builtinId="53" customBuiltin="1"/>
     <cellStyle name="Good" xfId="6" builtinId="26" customBuiltin="1"/>
     <cellStyle name="Heading 1" xfId="2" builtinId="16" customBuiltin="1"/>
@@ -1326,7 +1369,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H547"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
@@ -12236,327 +12279,824 @@
         <v>98</v>
       </c>
       <c r="B420" s="3">
-        <v>1871950730</v>
+        <f>SUMIFS('II PD'!C:C,'II PD'!A:A,'Budget 3 Juni 2024'!A420)</f>
+        <v>873740000</v>
       </c>
       <c r="C420" s="3">
-        <v>1871950730</v>
+        <f>SUMIFS('II PD'!D:D,'II PD'!A:A,'Budget 3 Juni 2024'!A420)</f>
+        <v>436870000</v>
       </c>
       <c r="D420" s="3">
-        <v>404935052</v>
+        <f>SUMIFS('II PD'!E:E,'II PD'!A:A,'Budget 3 Juni 2024'!A420)</f>
+        <v>404360000</v>
       </c>
       <c r="E420" s="3">
-        <v>78896778</v>
+        <f>SUMIFS('II PD'!F:F,'II PD'!A:A,'Budget 3 Juni 2024'!A420)</f>
+        <v>35605052</v>
       </c>
       <c r="F420" s="3">
-        <v>483831830</v>
+        <f>SUMIFS('II PD'!G:G,'II PD'!A:A,'Budget 3 Juni 2024'!A420)</f>
+        <v>439965052</v>
       </c>
       <c r="G420" s="3">
-        <v>1388118900</v>
+        <f>SUMIFS('II PD'!H:H,'II PD'!A:A,'Budget 3 Juni 2024'!A420)</f>
+        <v>-3095052</v>
       </c>
       <c r="H420" s="3">
-        <v>0</v>
+        <f>SUMIFS('II PD'!I:I,'II PD'!A:A,'Budget 3 Juni 2024'!A420)</f>
+        <v>436870000</v>
       </c>
     </row>
     <row r="421" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A421" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="B421" s="3"/>
-      <c r="C421" s="3"/>
-      <c r="D421" s="3"/>
-      <c r="E421" s="3"/>
-      <c r="F421" s="3"/>
-      <c r="G421" s="3"/>
-      <c r="H421" s="3"/>
+      <c r="B421" s="3">
+        <f>SUMIFS('II PD'!C:C,'II PD'!A:A,'Budget 3 Juni 2024'!A421)</f>
+        <v>0</v>
+      </c>
+      <c r="C421" s="3">
+        <f>SUMIFS('II PD'!D:D,'II PD'!A:A,'Budget 3 Juni 2024'!A421)</f>
+        <v>0</v>
+      </c>
+      <c r="D421" s="3">
+        <f>SUMIFS('II PD'!E:E,'II PD'!A:A,'Budget 3 Juni 2024'!A421)</f>
+        <v>0</v>
+      </c>
+      <c r="E421" s="3">
+        <f>SUMIFS('II PD'!F:F,'II PD'!A:A,'Budget 3 Juni 2024'!A421)</f>
+        <v>0</v>
+      </c>
+      <c r="F421" s="3">
+        <f>SUMIFS('II PD'!G:G,'II PD'!A:A,'Budget 3 Juni 2024'!A421)</f>
+        <v>0</v>
+      </c>
+      <c r="G421" s="3">
+        <f>SUMIFS('II PD'!H:H,'II PD'!A:A,'Budget 3 Juni 2024'!A421)</f>
+        <v>0</v>
+      </c>
+      <c r="H421" s="3">
+        <f>SUMIFS('II PD'!I:I,'II PD'!A:A,'Budget 3 Juni 2024'!A421)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="422" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A422" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="B422" s="3"/>
-      <c r="C422" s="3"/>
-      <c r="D422" s="3"/>
-      <c r="E422" s="3"/>
-      <c r="F422" s="3"/>
-      <c r="G422" s="3"/>
-      <c r="H422" s="3"/>
+      <c r="B422" s="3">
+        <f>SUMIFS('II PD'!C:C,'II PD'!A:A,'Budget 3 Juni 2024'!A422)</f>
+        <v>0</v>
+      </c>
+      <c r="C422" s="3">
+        <f>SUMIFS('II PD'!D:D,'II PD'!A:A,'Budget 3 Juni 2024'!A422)</f>
+        <v>0</v>
+      </c>
+      <c r="D422" s="3">
+        <f>SUMIFS('II PD'!E:E,'II PD'!A:A,'Budget 3 Juni 2024'!A422)</f>
+        <v>0</v>
+      </c>
+      <c r="E422" s="3">
+        <f>SUMIFS('II PD'!F:F,'II PD'!A:A,'Budget 3 Juni 2024'!A422)</f>
+        <v>0</v>
+      </c>
+      <c r="F422" s="3">
+        <f>SUMIFS('II PD'!G:G,'II PD'!A:A,'Budget 3 Juni 2024'!A422)</f>
+        <v>0</v>
+      </c>
+      <c r="G422" s="3">
+        <f>SUMIFS('II PD'!H:H,'II PD'!A:A,'Budget 3 Juni 2024'!A422)</f>
+        <v>0</v>
+      </c>
+      <c r="H422" s="3">
+        <f>SUMIFS('II PD'!I:I,'II PD'!A:A,'Budget 3 Juni 2024'!A422)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="423" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A423" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="B423" s="3"/>
-      <c r="C423" s="3"/>
-      <c r="D423" s="3"/>
-      <c r="E423" s="3"/>
-      <c r="F423" s="3"/>
-      <c r="G423" s="3"/>
-      <c r="H423" s="3"/>
+      <c r="B423" s="3">
+        <f>SUMIFS('II PD'!C:C,'II PD'!A:A,'Budget 3 Juni 2024'!A423)</f>
+        <v>0</v>
+      </c>
+      <c r="C423" s="3">
+        <f>SUMIFS('II PD'!D:D,'II PD'!A:A,'Budget 3 Juni 2024'!A423)</f>
+        <v>0</v>
+      </c>
+      <c r="D423" s="3">
+        <f>SUMIFS('II PD'!E:E,'II PD'!A:A,'Budget 3 Juni 2024'!A423)</f>
+        <v>0</v>
+      </c>
+      <c r="E423" s="3">
+        <f>SUMIFS('II PD'!F:F,'II PD'!A:A,'Budget 3 Juni 2024'!A423)</f>
+        <v>0</v>
+      </c>
+      <c r="F423" s="3">
+        <f>SUMIFS('II PD'!G:G,'II PD'!A:A,'Budget 3 Juni 2024'!A423)</f>
+        <v>0</v>
+      </c>
+      <c r="G423" s="3">
+        <f>SUMIFS('II PD'!H:H,'II PD'!A:A,'Budget 3 Juni 2024'!A423)</f>
+        <v>0</v>
+      </c>
+      <c r="H423" s="3">
+        <f>SUMIFS('II PD'!I:I,'II PD'!A:A,'Budget 3 Juni 2024'!A423)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="424" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A424" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="B424" s="3"/>
-      <c r="C424" s="3"/>
-      <c r="D424" s="3"/>
-      <c r="E424" s="3"/>
-      <c r="F424" s="3"/>
-      <c r="G424" s="3"/>
-      <c r="H424" s="3"/>
+      <c r="B424" s="3">
+        <f>SUMIFS('II PD'!C:C,'II PD'!A:A,'Budget 3 Juni 2024'!A424)</f>
+        <v>0</v>
+      </c>
+      <c r="C424" s="3">
+        <f>SUMIFS('II PD'!D:D,'II PD'!A:A,'Budget 3 Juni 2024'!A424)</f>
+        <v>0</v>
+      </c>
+      <c r="D424" s="3">
+        <f>SUMIFS('II PD'!E:E,'II PD'!A:A,'Budget 3 Juni 2024'!A424)</f>
+        <v>0</v>
+      </c>
+      <c r="E424" s="3">
+        <f>SUMIFS('II PD'!F:F,'II PD'!A:A,'Budget 3 Juni 2024'!A424)</f>
+        <v>0</v>
+      </c>
+      <c r="F424" s="3">
+        <f>SUMIFS('II PD'!G:G,'II PD'!A:A,'Budget 3 Juni 2024'!A424)</f>
+        <v>0</v>
+      </c>
+      <c r="G424" s="3">
+        <f>SUMIFS('II PD'!H:H,'II PD'!A:A,'Budget 3 Juni 2024'!A424)</f>
+        <v>0</v>
+      </c>
+      <c r="H424" s="3">
+        <f>SUMIFS('II PD'!I:I,'II PD'!A:A,'Budget 3 Juni 2024'!A424)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="425" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A425" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="B425" s="3"/>
-      <c r="C425" s="3"/>
-      <c r="D425" s="3"/>
-      <c r="E425" s="3"/>
-      <c r="F425" s="3"/>
-      <c r="G425" s="3"/>
-      <c r="H425" s="3"/>
+      <c r="B425" s="3">
+        <f>SUMIFS('II PD'!C:C,'II PD'!A:A,'Budget 3 Juni 2024'!A425)</f>
+        <v>0</v>
+      </c>
+      <c r="C425" s="3">
+        <f>SUMIFS('II PD'!D:D,'II PD'!A:A,'Budget 3 Juni 2024'!A425)</f>
+        <v>0</v>
+      </c>
+      <c r="D425" s="3">
+        <f>SUMIFS('II PD'!E:E,'II PD'!A:A,'Budget 3 Juni 2024'!A425)</f>
+        <v>0</v>
+      </c>
+      <c r="E425" s="3">
+        <f>SUMIFS('II PD'!F:F,'II PD'!A:A,'Budget 3 Juni 2024'!A425)</f>
+        <v>0</v>
+      </c>
+      <c r="F425" s="3">
+        <f>SUMIFS('II PD'!G:G,'II PD'!A:A,'Budget 3 Juni 2024'!A425)</f>
+        <v>0</v>
+      </c>
+      <c r="G425" s="3">
+        <f>SUMIFS('II PD'!H:H,'II PD'!A:A,'Budget 3 Juni 2024'!A425)</f>
+        <v>0</v>
+      </c>
+      <c r="H425" s="3">
+        <f>SUMIFS('II PD'!I:I,'II PD'!A:A,'Budget 3 Juni 2024'!A425)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="426" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A426" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="B426" s="3"/>
-      <c r="C426" s="3"/>
-      <c r="D426" s="3"/>
-      <c r="E426" s="3"/>
-      <c r="F426" s="3"/>
-      <c r="G426" s="3"/>
-      <c r="H426" s="3"/>
+      <c r="B426" s="3">
+        <f>SUMIFS('II PD'!C:C,'II PD'!A:A,'Budget 3 Juni 2024'!A426)</f>
+        <v>0</v>
+      </c>
+      <c r="C426" s="3">
+        <f>SUMIFS('II PD'!D:D,'II PD'!A:A,'Budget 3 Juni 2024'!A426)</f>
+        <v>0</v>
+      </c>
+      <c r="D426" s="3">
+        <f>SUMIFS('II PD'!E:E,'II PD'!A:A,'Budget 3 Juni 2024'!A426)</f>
+        <v>0</v>
+      </c>
+      <c r="E426" s="3">
+        <f>SUMIFS('II PD'!F:F,'II PD'!A:A,'Budget 3 Juni 2024'!A426)</f>
+        <v>0</v>
+      </c>
+      <c r="F426" s="3">
+        <f>SUMIFS('II PD'!G:G,'II PD'!A:A,'Budget 3 Juni 2024'!A426)</f>
+        <v>0</v>
+      </c>
+      <c r="G426" s="3">
+        <f>SUMIFS('II PD'!H:H,'II PD'!A:A,'Budget 3 Juni 2024'!A426)</f>
+        <v>0</v>
+      </c>
+      <c r="H426" s="3">
+        <f>SUMIFS('II PD'!I:I,'II PD'!A:A,'Budget 3 Juni 2024'!A426)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="427" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A427" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="B427" s="3"/>
-      <c r="C427" s="3"/>
-      <c r="D427" s="3"/>
-      <c r="E427" s="3"/>
-      <c r="F427" s="3"/>
-      <c r="G427" s="3"/>
-      <c r="H427" s="3"/>
+      <c r="B427" s="3">
+        <f>SUMIFS('II PD'!C:C,'II PD'!A:A,'Budget 3 Juni 2024'!A427)</f>
+        <v>0</v>
+      </c>
+      <c r="C427" s="3">
+        <f>SUMIFS('II PD'!D:D,'II PD'!A:A,'Budget 3 Juni 2024'!A427)</f>
+        <v>0</v>
+      </c>
+      <c r="D427" s="3">
+        <f>SUMIFS('II PD'!E:E,'II PD'!A:A,'Budget 3 Juni 2024'!A427)</f>
+        <v>0</v>
+      </c>
+      <c r="E427" s="3">
+        <f>SUMIFS('II PD'!F:F,'II PD'!A:A,'Budget 3 Juni 2024'!A427)</f>
+        <v>0</v>
+      </c>
+      <c r="F427" s="3">
+        <f>SUMIFS('II PD'!G:G,'II PD'!A:A,'Budget 3 Juni 2024'!A427)</f>
+        <v>0</v>
+      </c>
+      <c r="G427" s="3">
+        <f>SUMIFS('II PD'!H:H,'II PD'!A:A,'Budget 3 Juni 2024'!A427)</f>
+        <v>0</v>
+      </c>
+      <c r="H427" s="3">
+        <f>SUMIFS('II PD'!I:I,'II PD'!A:A,'Budget 3 Juni 2024'!A427)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="428" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A428" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="B428" s="3"/>
-      <c r="C428" s="3"/>
-      <c r="D428" s="3"/>
-      <c r="E428" s="3"/>
-      <c r="F428" s="3"/>
-      <c r="G428" s="3"/>
-      <c r="H428" s="3"/>
+      <c r="B428" s="3">
+        <f>SUMIFS('II PD'!C:C,'II PD'!A:A,'Budget 3 Juni 2024'!A428)</f>
+        <v>0</v>
+      </c>
+      <c r="C428" s="3">
+        <f>SUMIFS('II PD'!D:D,'II PD'!A:A,'Budget 3 Juni 2024'!A428)</f>
+        <v>0</v>
+      </c>
+      <c r="D428" s="3">
+        <f>SUMIFS('II PD'!E:E,'II PD'!A:A,'Budget 3 Juni 2024'!A428)</f>
+        <v>0</v>
+      </c>
+      <c r="E428" s="3">
+        <f>SUMIFS('II PD'!F:F,'II PD'!A:A,'Budget 3 Juni 2024'!A428)</f>
+        <v>0</v>
+      </c>
+      <c r="F428" s="3">
+        <f>SUMIFS('II PD'!G:G,'II PD'!A:A,'Budget 3 Juni 2024'!A428)</f>
+        <v>0</v>
+      </c>
+      <c r="G428" s="3">
+        <f>SUMIFS('II PD'!H:H,'II PD'!A:A,'Budget 3 Juni 2024'!A428)</f>
+        <v>0</v>
+      </c>
+      <c r="H428" s="3">
+        <f>SUMIFS('II PD'!I:I,'II PD'!A:A,'Budget 3 Juni 2024'!A428)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="429" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A429" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="B429" s="3"/>
-      <c r="C429" s="3"/>
-      <c r="D429" s="3"/>
-      <c r="E429" s="3"/>
-      <c r="F429" s="3"/>
-      <c r="G429" s="3"/>
-      <c r="H429" s="3"/>
+      <c r="B429" s="3">
+        <f>SUMIFS('II PD'!C:C,'II PD'!A:A,'Budget 3 Juni 2024'!A429)</f>
+        <v>0</v>
+      </c>
+      <c r="C429" s="3">
+        <f>SUMIFS('II PD'!D:D,'II PD'!A:A,'Budget 3 Juni 2024'!A429)</f>
+        <v>0</v>
+      </c>
+      <c r="D429" s="3">
+        <f>SUMIFS('II PD'!E:E,'II PD'!A:A,'Budget 3 Juni 2024'!A429)</f>
+        <v>0</v>
+      </c>
+      <c r="E429" s="3">
+        <f>SUMIFS('II PD'!F:F,'II PD'!A:A,'Budget 3 Juni 2024'!A429)</f>
+        <v>0</v>
+      </c>
+      <c r="F429" s="3">
+        <f>SUMIFS('II PD'!G:G,'II PD'!A:A,'Budget 3 Juni 2024'!A429)</f>
+        <v>0</v>
+      </c>
+      <c r="G429" s="3">
+        <f>SUMIFS('II PD'!H:H,'II PD'!A:A,'Budget 3 Juni 2024'!A429)</f>
+        <v>0</v>
+      </c>
+      <c r="H429" s="3">
+        <f>SUMIFS('II PD'!I:I,'II PD'!A:A,'Budget 3 Juni 2024'!A429)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="430" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A430" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="B430" s="3"/>
-      <c r="C430" s="3"/>
-      <c r="D430" s="3"/>
-      <c r="E430" s="3"/>
-      <c r="F430" s="3"/>
-      <c r="G430" s="3"/>
-      <c r="H430" s="3"/>
+      <c r="B430" s="3">
+        <f>SUMIFS('II PD'!C:C,'II PD'!A:A,'Budget 3 Juni 2024'!A430)</f>
+        <v>0</v>
+      </c>
+      <c r="C430" s="3">
+        <f>SUMIFS('II PD'!D:D,'II PD'!A:A,'Budget 3 Juni 2024'!A430)</f>
+        <v>0</v>
+      </c>
+      <c r="D430" s="3">
+        <f>SUMIFS('II PD'!E:E,'II PD'!A:A,'Budget 3 Juni 2024'!A430)</f>
+        <v>0</v>
+      </c>
+      <c r="E430" s="3">
+        <f>SUMIFS('II PD'!F:F,'II PD'!A:A,'Budget 3 Juni 2024'!A430)</f>
+        <v>0</v>
+      </c>
+      <c r="F430" s="3">
+        <f>SUMIFS('II PD'!G:G,'II PD'!A:A,'Budget 3 Juni 2024'!A430)</f>
+        <v>0</v>
+      </c>
+      <c r="G430" s="3">
+        <f>SUMIFS('II PD'!H:H,'II PD'!A:A,'Budget 3 Juni 2024'!A430)</f>
+        <v>0</v>
+      </c>
+      <c r="H430" s="3">
+        <f>SUMIFS('II PD'!I:I,'II PD'!A:A,'Budget 3 Juni 2024'!A430)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="431" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A431" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="B431" s="3"/>
-      <c r="C431" s="3"/>
-      <c r="D431" s="3"/>
-      <c r="E431" s="3"/>
-      <c r="F431" s="3"/>
-      <c r="G431" s="3"/>
-      <c r="H431" s="3"/>
+      <c r="B431" s="3">
+        <f>SUMIFS('II PD'!C:C,'II PD'!A:A,'Budget 3 Juni 2024'!A431)</f>
+        <v>0</v>
+      </c>
+      <c r="C431" s="3">
+        <f>SUMIFS('II PD'!D:D,'II PD'!A:A,'Budget 3 Juni 2024'!A431)</f>
+        <v>0</v>
+      </c>
+      <c r="D431" s="3">
+        <f>SUMIFS('II PD'!E:E,'II PD'!A:A,'Budget 3 Juni 2024'!A431)</f>
+        <v>0</v>
+      </c>
+      <c r="E431" s="3">
+        <f>SUMIFS('II PD'!F:F,'II PD'!A:A,'Budget 3 Juni 2024'!A431)</f>
+        <v>0</v>
+      </c>
+      <c r="F431" s="3">
+        <f>SUMIFS('II PD'!G:G,'II PD'!A:A,'Budget 3 Juni 2024'!A431)</f>
+        <v>0</v>
+      </c>
+      <c r="G431" s="3">
+        <f>SUMIFS('II PD'!H:H,'II PD'!A:A,'Budget 3 Juni 2024'!A431)</f>
+        <v>0</v>
+      </c>
+      <c r="H431" s="3">
+        <f>SUMIFS('II PD'!I:I,'II PD'!A:A,'Budget 3 Juni 2024'!A431)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="432" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A432" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="B432" s="3"/>
-      <c r="C432" s="3"/>
-      <c r="D432" s="3"/>
-      <c r="E432" s="3"/>
-      <c r="F432" s="3"/>
-      <c r="G432" s="3"/>
-      <c r="H432" s="3"/>
+      <c r="B432" s="3">
+        <f>SUMIFS('II PD'!C:C,'II PD'!A:A,'Budget 3 Juni 2024'!A432)</f>
+        <v>0</v>
+      </c>
+      <c r="C432" s="3">
+        <f>SUMIFS('II PD'!D:D,'II PD'!A:A,'Budget 3 Juni 2024'!A432)</f>
+        <v>0</v>
+      </c>
+      <c r="D432" s="3">
+        <f>SUMIFS('II PD'!E:E,'II PD'!A:A,'Budget 3 Juni 2024'!A432)</f>
+        <v>0</v>
+      </c>
+      <c r="E432" s="3">
+        <f>SUMIFS('II PD'!F:F,'II PD'!A:A,'Budget 3 Juni 2024'!A432)</f>
+        <v>0</v>
+      </c>
+      <c r="F432" s="3">
+        <f>SUMIFS('II PD'!G:G,'II PD'!A:A,'Budget 3 Juni 2024'!A432)</f>
+        <v>0</v>
+      </c>
+      <c r="G432" s="3">
+        <f>SUMIFS('II PD'!H:H,'II PD'!A:A,'Budget 3 Juni 2024'!A432)</f>
+        <v>0</v>
+      </c>
+      <c r="H432" s="3">
+        <f>SUMIFS('II PD'!I:I,'II PD'!A:A,'Budget 3 Juni 2024'!A432)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="433" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A433" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="B433" s="3"/>
-      <c r="C433" s="3"/>
-      <c r="D433" s="3"/>
-      <c r="E433" s="3"/>
-      <c r="F433" s="3"/>
-      <c r="G433" s="3"/>
-      <c r="H433" s="3"/>
+      <c r="B433" s="3">
+        <f>SUMIFS('II PD'!C:C,'II PD'!A:A,'Budget 3 Juni 2024'!A433)</f>
+        <v>0</v>
+      </c>
+      <c r="C433" s="3">
+        <f>SUMIFS('II PD'!D:D,'II PD'!A:A,'Budget 3 Juni 2024'!A433)</f>
+        <v>0</v>
+      </c>
+      <c r="D433" s="3">
+        <f>SUMIFS('II PD'!E:E,'II PD'!A:A,'Budget 3 Juni 2024'!A433)</f>
+        <v>0</v>
+      </c>
+      <c r="E433" s="3">
+        <f>SUMIFS('II PD'!F:F,'II PD'!A:A,'Budget 3 Juni 2024'!A433)</f>
+        <v>0</v>
+      </c>
+      <c r="F433" s="3">
+        <f>SUMIFS('II PD'!G:G,'II PD'!A:A,'Budget 3 Juni 2024'!A433)</f>
+        <v>0</v>
+      </c>
+      <c r="G433" s="3">
+        <f>SUMIFS('II PD'!H:H,'II PD'!A:A,'Budget 3 Juni 2024'!A433)</f>
+        <v>0</v>
+      </c>
+      <c r="H433" s="3">
+        <f>SUMIFS('II PD'!I:I,'II PD'!A:A,'Budget 3 Juni 2024'!A433)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="434" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A434" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="B434" s="3"/>
-      <c r="C434" s="3"/>
-      <c r="D434" s="3"/>
-      <c r="E434" s="3"/>
-      <c r="F434" s="3"/>
-      <c r="G434" s="3"/>
-      <c r="H434" s="3"/>
+      <c r="B434" s="3">
+        <f>SUMIFS('II PD'!C:C,'II PD'!A:A,'Budget 3 Juni 2024'!A434)</f>
+        <v>0</v>
+      </c>
+      <c r="C434" s="3">
+        <f>SUMIFS('II PD'!D:D,'II PD'!A:A,'Budget 3 Juni 2024'!A434)</f>
+        <v>0</v>
+      </c>
+      <c r="D434" s="3">
+        <f>SUMIFS('II PD'!E:E,'II PD'!A:A,'Budget 3 Juni 2024'!A434)</f>
+        <v>0</v>
+      </c>
+      <c r="E434" s="3">
+        <f>SUMIFS('II PD'!F:F,'II PD'!A:A,'Budget 3 Juni 2024'!A434)</f>
+        <v>0</v>
+      </c>
+      <c r="F434" s="3">
+        <f>SUMIFS('II PD'!G:G,'II PD'!A:A,'Budget 3 Juni 2024'!A434)</f>
+        <v>0</v>
+      </c>
+      <c r="G434" s="3">
+        <f>SUMIFS('II PD'!H:H,'II PD'!A:A,'Budget 3 Juni 2024'!A434)</f>
+        <v>0</v>
+      </c>
+      <c r="H434" s="3">
+        <f>SUMIFS('II PD'!I:I,'II PD'!A:A,'Budget 3 Juni 2024'!A434)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="435" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A435" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="B435" s="3"/>
-      <c r="C435" s="3"/>
-      <c r="D435" s="3"/>
-      <c r="E435" s="3"/>
-      <c r="F435" s="3"/>
-      <c r="G435" s="3"/>
-      <c r="H435" s="3"/>
+      <c r="B435" s="3">
+        <f>SUMIFS('II PD'!C:C,'II PD'!A:A,'Budget 3 Juni 2024'!A435)</f>
+        <v>0</v>
+      </c>
+      <c r="C435" s="3">
+        <f>SUMIFS('II PD'!D:D,'II PD'!A:A,'Budget 3 Juni 2024'!A435)</f>
+        <v>0</v>
+      </c>
+      <c r="D435" s="3">
+        <f>SUMIFS('II PD'!E:E,'II PD'!A:A,'Budget 3 Juni 2024'!A435)</f>
+        <v>0</v>
+      </c>
+      <c r="E435" s="3">
+        <f>SUMIFS('II PD'!F:F,'II PD'!A:A,'Budget 3 Juni 2024'!A435)</f>
+        <v>0</v>
+      </c>
+      <c r="F435" s="3">
+        <f>SUMIFS('II PD'!G:G,'II PD'!A:A,'Budget 3 Juni 2024'!A435)</f>
+        <v>0</v>
+      </c>
+      <c r="G435" s="3">
+        <f>SUMIFS('II PD'!H:H,'II PD'!A:A,'Budget 3 Juni 2024'!A435)</f>
+        <v>0</v>
+      </c>
+      <c r="H435" s="3">
+        <f>SUMIFS('II PD'!I:I,'II PD'!A:A,'Budget 3 Juni 2024'!A435)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="436" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A436" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="B436" s="3"/>
-      <c r="C436" s="3"/>
-      <c r="D436" s="3"/>
-      <c r="E436" s="3"/>
-      <c r="F436" s="3"/>
-      <c r="G436" s="3"/>
-      <c r="H436" s="3"/>
+      <c r="B436" s="3">
+        <f>SUMIFS('II PD'!C:C,'II PD'!A:A,'Budget 3 Juni 2024'!A436)</f>
+        <v>0</v>
+      </c>
+      <c r="C436" s="3">
+        <f>SUMIFS('II PD'!D:D,'II PD'!A:A,'Budget 3 Juni 2024'!A436)</f>
+        <v>0</v>
+      </c>
+      <c r="D436" s="3">
+        <f>SUMIFS('II PD'!E:E,'II PD'!A:A,'Budget 3 Juni 2024'!A436)</f>
+        <v>0</v>
+      </c>
+      <c r="E436" s="3">
+        <f>SUMIFS('II PD'!F:F,'II PD'!A:A,'Budget 3 Juni 2024'!A436)</f>
+        <v>0</v>
+      </c>
+      <c r="F436" s="3">
+        <f>SUMIFS('II PD'!G:G,'II PD'!A:A,'Budget 3 Juni 2024'!A436)</f>
+        <v>0</v>
+      </c>
+      <c r="G436" s="3">
+        <f>SUMIFS('II PD'!H:H,'II PD'!A:A,'Budget 3 Juni 2024'!A436)</f>
+        <v>0</v>
+      </c>
+      <c r="H436" s="3">
+        <f>SUMIFS('II PD'!I:I,'II PD'!A:A,'Budget 3 Juni 2024'!A436)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="437" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A437" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="B437" s="3"/>
-      <c r="C437" s="3"/>
-      <c r="D437" s="3"/>
-      <c r="E437" s="3"/>
-      <c r="F437" s="3"/>
-      <c r="G437" s="3"/>
-      <c r="H437" s="3"/>
+      <c r="B437" s="3">
+        <f>SUMIFS('II PD'!C:C,'II PD'!A:A,'Budget 3 Juni 2024'!A437)</f>
+        <v>474786000</v>
+      </c>
+      <c r="C437" s="3">
+        <f>SUMIFS('II PD'!D:D,'II PD'!A:A,'Budget 3 Juni 2024'!A437)</f>
+        <v>237393000</v>
+      </c>
+      <c r="D437" s="3">
+        <f>SUMIFS('II PD'!E:E,'II PD'!A:A,'Budget 3 Juni 2024'!A437)</f>
+        <v>0</v>
+      </c>
+      <c r="E437" s="3">
+        <f>SUMIFS('II PD'!F:F,'II PD'!A:A,'Budget 3 Juni 2024'!A437)</f>
+        <v>0</v>
+      </c>
+      <c r="F437" s="3">
+        <f>SUMIFS('II PD'!G:G,'II PD'!A:A,'Budget 3 Juni 2024'!A437)</f>
+        <v>0</v>
+      </c>
+      <c r="G437" s="3">
+        <f>SUMIFS('II PD'!H:H,'II PD'!A:A,'Budget 3 Juni 2024'!A437)</f>
+        <v>237393000</v>
+      </c>
+      <c r="H437" s="3">
+        <f>SUMIFS('II PD'!I:I,'II PD'!A:A,'Budget 3 Juni 2024'!A437)</f>
+        <v>237393000</v>
+      </c>
     </row>
     <row r="438" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A438" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="B438" s="3"/>
-      <c r="C438" s="3"/>
-      <c r="D438" s="3"/>
-      <c r="E438" s="3"/>
-      <c r="F438" s="3"/>
-      <c r="G438" s="3"/>
-      <c r="H438" s="3"/>
+      <c r="B438" s="3">
+        <f>SUMIFS('II PD'!C:C,'II PD'!A:A,'Budget 3 Juni 2024'!A438)</f>
+        <v>208425000</v>
+      </c>
+      <c r="C438" s="3">
+        <f>SUMIFS('II PD'!D:D,'II PD'!A:A,'Budget 3 Juni 2024'!A438)</f>
+        <v>104212500</v>
+      </c>
+      <c r="D438" s="3">
+        <f>SUMIFS('II PD'!E:E,'II PD'!A:A,'Budget 3 Juni 2024'!A438)</f>
+        <v>0</v>
+      </c>
+      <c r="E438" s="3">
+        <f>SUMIFS('II PD'!F:F,'II PD'!A:A,'Budget 3 Juni 2024'!A438)</f>
+        <v>0</v>
+      </c>
+      <c r="F438" s="3">
+        <f>SUMIFS('II PD'!G:G,'II PD'!A:A,'Budget 3 Juni 2024'!A438)</f>
+        <v>0</v>
+      </c>
+      <c r="G438" s="3">
+        <f>SUMIFS('II PD'!H:H,'II PD'!A:A,'Budget 3 Juni 2024'!A438)</f>
+        <v>104212500</v>
+      </c>
+      <c r="H438" s="3">
+        <f>SUMIFS('II PD'!I:I,'II PD'!A:A,'Budget 3 Juni 2024'!A438)</f>
+        <v>104212500</v>
+      </c>
     </row>
     <row r="439" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A439" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="B439" s="3"/>
-      <c r="C439" s="3"/>
-      <c r="D439" s="3"/>
-      <c r="E439" s="3"/>
-      <c r="F439" s="3"/>
-      <c r="G439" s="3"/>
-      <c r="H439" s="3"/>
+      <c r="B439" s="3">
+        <f>SUMIFS('II PD'!C:C,'II PD'!A:A,'Budget 3 Juni 2024'!A439)</f>
+        <v>20000000</v>
+      </c>
+      <c r="C439" s="3">
+        <f>SUMIFS('II PD'!D:D,'II PD'!A:A,'Budget 3 Juni 2024'!A439)</f>
+        <v>13970000</v>
+      </c>
+      <c r="D439" s="3">
+        <f>SUMIFS('II PD'!E:E,'II PD'!A:A,'Budget 3 Juni 2024'!A439)</f>
+        <v>13970000</v>
+      </c>
+      <c r="E439" s="3">
+        <f>SUMIFS('II PD'!F:F,'II PD'!A:A,'Budget 3 Juni 2024'!A439)</f>
+        <v>0</v>
+      </c>
+      <c r="F439" s="3">
+        <f>SUMIFS('II PD'!G:G,'II PD'!A:A,'Budget 3 Juni 2024'!A439)</f>
+        <v>13970000</v>
+      </c>
+      <c r="G439" s="3">
+        <f>SUMIFS('II PD'!H:H,'II PD'!A:A,'Budget 3 Juni 2024'!A439)</f>
+        <v>0</v>
+      </c>
+      <c r="H439" s="3">
+        <f>SUMIFS('II PD'!I:I,'II PD'!A:A,'Budget 3 Juni 2024'!A439)</f>
+        <v>6030000</v>
+      </c>
     </row>
     <row r="440" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A440" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="B440" s="3"/>
-      <c r="C440" s="3"/>
-      <c r="D440" s="3"/>
-      <c r="E440" s="3"/>
-      <c r="F440" s="3"/>
-      <c r="G440" s="3"/>
-      <c r="H440" s="3"/>
+      <c r="B440" s="3">
+        <f>SUMIFS('II PD'!C:C,'II PD'!A:A,'Budget 3 Juni 2024'!A440)</f>
+        <v>220000000</v>
+      </c>
+      <c r="C440" s="3">
+        <f>SUMIFS('II PD'!D:D,'II PD'!A:A,'Budget 3 Juni 2024'!A440)</f>
+        <v>110000000</v>
+      </c>
+      <c r="D440" s="3">
+        <f>SUMIFS('II PD'!E:E,'II PD'!A:A,'Budget 3 Juni 2024'!A440)</f>
+        <v>0</v>
+      </c>
+      <c r="E440" s="3">
+        <f>SUMIFS('II PD'!F:F,'II PD'!A:A,'Budget 3 Juni 2024'!A440)</f>
+        <v>29896778</v>
+      </c>
+      <c r="F440" s="3">
+        <f>SUMIFS('II PD'!G:G,'II PD'!A:A,'Budget 3 Juni 2024'!A440)</f>
+        <v>29896778</v>
+      </c>
+      <c r="G440" s="3">
+        <f>SUMIFS('II PD'!H:H,'II PD'!A:A,'Budget 3 Juni 2024'!A440)</f>
+        <v>80103222</v>
+      </c>
+      <c r="H440" s="3">
+        <f>SUMIFS('II PD'!I:I,'II PD'!A:A,'Budget 3 Juni 2024'!A440)</f>
+        <v>110000000</v>
+      </c>
     </row>
     <row r="441" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A441" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="B441" s="3"/>
-      <c r="C441" s="3"/>
-      <c r="D441" s="3"/>
-      <c r="E441" s="3"/>
-      <c r="F441" s="3"/>
-      <c r="G441" s="3"/>
-      <c r="H441" s="3"/>
+      <c r="B441" s="3">
+        <f>SUMIFS('II PD'!C:C,'II PD'!A:A,'Budget 3 Juni 2024'!A441)</f>
+        <v>75000000</v>
+      </c>
+      <c r="C441" s="3">
+        <f>SUMIFS('II PD'!D:D,'II PD'!A:A,'Budget 3 Juni 2024'!A441)</f>
+        <v>37500000</v>
+      </c>
+      <c r="D441" s="3">
+        <f>SUMIFS('II PD'!E:E,'II PD'!A:A,'Budget 3 Juni 2024'!A441)</f>
+        <v>0</v>
+      </c>
+      <c r="E441" s="3">
+        <f>SUMIFS('II PD'!F:F,'II PD'!A:A,'Budget 3 Juni 2024'!A441)</f>
+        <v>0</v>
+      </c>
+      <c r="F441" s="3">
+        <f>SUMIFS('II PD'!G:G,'II PD'!A:A,'Budget 3 Juni 2024'!A441)</f>
+        <v>0</v>
+      </c>
+      <c r="G441" s="3">
+        <f>SUMIFS('II PD'!H:H,'II PD'!A:A,'Budget 3 Juni 2024'!A441)</f>
+        <v>37500000</v>
+      </c>
+      <c r="H441" s="3">
+        <f>SUMIFS('II PD'!I:I,'II PD'!A:A,'Budget 3 Juni 2024'!A441)</f>
+        <v>37500000</v>
+      </c>
     </row>
     <row r="442" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A442" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="B442" s="3"/>
-      <c r="C442" s="3"/>
-      <c r="D442" s="3"/>
-      <c r="E442" s="3"/>
-      <c r="F442" s="3"/>
-      <c r="G442" s="3"/>
-      <c r="H442" s="3"/>
+      <c r="B442" s="3">
+        <f>SUMIFS('II PD'!C:C,'II PD'!A:A,'Budget 3 Juni 2024'!A442)</f>
+        <v>0</v>
+      </c>
+      <c r="C442" s="3">
+        <f>SUMIFS('II PD'!D:D,'II PD'!A:A,'Budget 3 Juni 2024'!A442)</f>
+        <v>0</v>
+      </c>
+      <c r="D442" s="3">
+        <f>SUMIFS('II PD'!E:E,'II PD'!A:A,'Budget 3 Juni 2024'!A442)</f>
+        <v>0</v>
+      </c>
+      <c r="E442" s="3">
+        <f>SUMIFS('II PD'!F:F,'II PD'!A:A,'Budget 3 Juni 2024'!A442)</f>
+        <v>0</v>
+      </c>
+      <c r="F442" s="3">
+        <f>SUMIFS('II PD'!G:G,'II PD'!A:A,'Budget 3 Juni 2024'!A442)</f>
+        <v>0</v>
+      </c>
+      <c r="G442" s="3">
+        <f>SUMIFS('II PD'!H:H,'II PD'!A:A,'Budget 3 Juni 2024'!A442)</f>
+        <v>0</v>
+      </c>
+      <c r="H442" s="3">
+        <f>SUMIFS('II PD'!I:I,'II PD'!A:A,'Budget 3 Juni 2024'!A442)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="443" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A443" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="B443" s="3"/>
-      <c r="C443" s="3"/>
-      <c r="D443" s="3"/>
-      <c r="E443" s="3"/>
-      <c r="F443" s="3"/>
-      <c r="G443" s="3"/>
-      <c r="H443" s="3"/>
+      <c r="B443" s="3">
+        <f>SUMIFS('II PD'!C:C,'II PD'!A:A,'Budget 3 Juni 2024'!A443)</f>
+        <v>0</v>
+      </c>
+      <c r="C443" s="3">
+        <f>SUMIFS('II PD'!D:D,'II PD'!A:A,'Budget 3 Juni 2024'!A443)</f>
+        <v>0</v>
+      </c>
+      <c r="D443" s="3">
+        <f>SUMIFS('II PD'!E:E,'II PD'!A:A,'Budget 3 Juni 2024'!A443)</f>
+        <v>0</v>
+      </c>
+      <c r="E443" s="3">
+        <f>SUMIFS('II PD'!F:F,'II PD'!A:A,'Budget 3 Juni 2024'!A443)</f>
+        <v>0</v>
+      </c>
+      <c r="F443" s="3">
+        <f>SUMIFS('II PD'!G:G,'II PD'!A:A,'Budget 3 Juni 2024'!A443)</f>
+        <v>0</v>
+      </c>
+      <c r="G443" s="3">
+        <f>SUMIFS('II PD'!H:H,'II PD'!A:A,'Budget 3 Juni 2024'!A443)</f>
+        <v>0</v>
+      </c>
+      <c r="H443" s="3">
+        <f>SUMIFS('II PD'!I:I,'II PD'!A:A,'Budget 3 Juni 2024'!A443)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="444" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A444" s="1" t="s">
         <v>122</v>
       </c>
       <c r="B444" s="3">
+        <f>SUMIFS('II PD'!C:C,'II PD'!A:A,'Budget 3 Juni 2024'!A444)</f>
         <v>60000000</v>
       </c>
       <c r="C444" s="3">
-        <v>60000000</v>
+        <f>SUMIFS('II PD'!D:D,'II PD'!A:A,'Budget 3 Juni 2024'!A444)</f>
+        <v>30000000</v>
       </c>
       <c r="D444" s="3">
+        <f>SUMIFS('II PD'!E:E,'II PD'!A:A,'Budget 3 Juni 2024'!A444)</f>
         <v>9000000</v>
       </c>
       <c r="E444" s="3">
+        <f>SUMIFS('II PD'!F:F,'II PD'!A:A,'Budget 3 Juni 2024'!A444)</f>
         <v>0</v>
       </c>
       <c r="F444" s="3">
+        <f>SUMIFS('II PD'!G:G,'II PD'!A:A,'Budget 3 Juni 2024'!A444)</f>
         <v>9000000</v>
       </c>
       <c r="G444" s="3">
-        <v>51000000</v>
+        <f>SUMIFS('II PD'!H:H,'II PD'!A:A,'Budget 3 Juni 2024'!A444)</f>
+        <v>21000000</v>
       </c>
       <c r="H444" s="3">
-        <v>0</v>
+        <f>SUMIFS('II PD'!I:I,'II PD'!A:A,'Budget 3 Juni 2024'!A444)</f>
+        <v>30000000</v>
       </c>
     </row>
     <row r="445" spans="1:8" x14ac:dyDescent="0.45">
@@ -12564,377 +13104,923 @@
         <v>123</v>
       </c>
       <c r="B445" s="3">
+        <f>SUMIFS('II PD'!C:C,'II PD'!A:A,'Budget 3 Juni 2024'!A445)</f>
         <v>45150000</v>
       </c>
       <c r="C445" s="3">
-        <v>45150000</v>
+        <f>SUMIFS('II PD'!D:D,'II PD'!A:A,'Budget 3 Juni 2024'!A445)</f>
+        <v>22575000</v>
       </c>
       <c r="D445" s="3">
+        <f>SUMIFS('II PD'!E:E,'II PD'!A:A,'Budget 3 Juni 2024'!A445)</f>
         <v>6423200</v>
       </c>
       <c r="E445" s="3">
+        <f>SUMIFS('II PD'!F:F,'II PD'!A:A,'Budget 3 Juni 2024'!A445)</f>
         <v>6119400</v>
       </c>
       <c r="F445" s="3">
+        <f>SUMIFS('II PD'!G:G,'II PD'!A:A,'Budget 3 Juni 2024'!A445)</f>
         <v>12542600</v>
       </c>
       <c r="G445" s="3">
-        <v>32607400</v>
+        <f>SUMIFS('II PD'!H:H,'II PD'!A:A,'Budget 3 Juni 2024'!A445)</f>
+        <v>10032400</v>
       </c>
       <c r="H445" s="3">
-        <v>0</v>
+        <f>SUMIFS('II PD'!I:I,'II PD'!A:A,'Budget 3 Juni 2024'!A445)</f>
+        <v>22575000</v>
       </c>
     </row>
     <row r="446" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A446" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="B446" s="3"/>
-      <c r="C446" s="3"/>
-      <c r="D446" s="3"/>
-      <c r="E446" s="3"/>
-      <c r="F446" s="3"/>
-      <c r="G446" s="3"/>
-      <c r="H446" s="3"/>
+      <c r="B446" s="3">
+        <f>SUMIFS('II PD'!C:C,'II PD'!A:A,'Budget 3 Juni 2024'!A446)</f>
+        <v>0</v>
+      </c>
+      <c r="C446" s="3">
+        <f>SUMIFS('II PD'!D:D,'II PD'!A:A,'Budget 3 Juni 2024'!A446)</f>
+        <v>0</v>
+      </c>
+      <c r="D446" s="3">
+        <f>SUMIFS('II PD'!E:E,'II PD'!A:A,'Budget 3 Juni 2024'!A446)</f>
+        <v>0</v>
+      </c>
+      <c r="E446" s="3">
+        <f>SUMIFS('II PD'!F:F,'II PD'!A:A,'Budget 3 Juni 2024'!A446)</f>
+        <v>0</v>
+      </c>
+      <c r="F446" s="3">
+        <f>SUMIFS('II PD'!G:G,'II PD'!A:A,'Budget 3 Juni 2024'!A446)</f>
+        <v>0</v>
+      </c>
+      <c r="G446" s="3">
+        <f>SUMIFS('II PD'!H:H,'II PD'!A:A,'Budget 3 Juni 2024'!A446)</f>
+        <v>0</v>
+      </c>
+      <c r="H446" s="3">
+        <f>SUMIFS('II PD'!I:I,'II PD'!A:A,'Budget 3 Juni 2024'!A446)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="447" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A447" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="B447" s="3"/>
-      <c r="C447" s="3"/>
-      <c r="D447" s="3"/>
-      <c r="E447" s="3"/>
-      <c r="F447" s="3"/>
-      <c r="G447" s="3"/>
-      <c r="H447" s="3"/>
+      <c r="B447" s="3">
+        <f>SUMIFS('II PD'!C:C,'II PD'!A:A,'Budget 3 Juni 2024'!A447)</f>
+        <v>0</v>
+      </c>
+      <c r="C447" s="3">
+        <f>SUMIFS('II PD'!D:D,'II PD'!A:A,'Budget 3 Juni 2024'!A447)</f>
+        <v>0</v>
+      </c>
+      <c r="D447" s="3">
+        <f>SUMIFS('II PD'!E:E,'II PD'!A:A,'Budget 3 Juni 2024'!A447)</f>
+        <v>0</v>
+      </c>
+      <c r="E447" s="3">
+        <f>SUMIFS('II PD'!F:F,'II PD'!A:A,'Budget 3 Juni 2024'!A447)</f>
+        <v>0</v>
+      </c>
+      <c r="F447" s="3">
+        <f>SUMIFS('II PD'!G:G,'II PD'!A:A,'Budget 3 Juni 2024'!A447)</f>
+        <v>0</v>
+      </c>
+      <c r="G447" s="3">
+        <f>SUMIFS('II PD'!H:H,'II PD'!A:A,'Budget 3 Juni 2024'!A447)</f>
+        <v>0</v>
+      </c>
+      <c r="H447" s="3">
+        <f>SUMIFS('II PD'!I:I,'II PD'!A:A,'Budget 3 Juni 2024'!A447)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="448" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A448" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="B448" s="3"/>
-      <c r="C448" s="3"/>
-      <c r="D448" s="3"/>
-      <c r="E448" s="3"/>
-      <c r="F448" s="3"/>
-      <c r="G448" s="3"/>
-      <c r="H448" s="3"/>
+      <c r="B448" s="3">
+        <f>SUMIFS('II PD'!C:C,'II PD'!A:A,'Budget 3 Juni 2024'!A448)</f>
+        <v>0</v>
+      </c>
+      <c r="C448" s="3">
+        <f>SUMIFS('II PD'!D:D,'II PD'!A:A,'Budget 3 Juni 2024'!A448)</f>
+        <v>0</v>
+      </c>
+      <c r="D448" s="3">
+        <f>SUMIFS('II PD'!E:E,'II PD'!A:A,'Budget 3 Juni 2024'!A448)</f>
+        <v>0</v>
+      </c>
+      <c r="E448" s="3">
+        <f>SUMIFS('II PD'!F:F,'II PD'!A:A,'Budget 3 Juni 2024'!A448)</f>
+        <v>0</v>
+      </c>
+      <c r="F448" s="3">
+        <f>SUMIFS('II PD'!G:G,'II PD'!A:A,'Budget 3 Juni 2024'!A448)</f>
+        <v>0</v>
+      </c>
+      <c r="G448" s="3">
+        <f>SUMIFS('II PD'!H:H,'II PD'!A:A,'Budget 3 Juni 2024'!A448)</f>
+        <v>0</v>
+      </c>
+      <c r="H448" s="3">
+        <f>SUMIFS('II PD'!I:I,'II PD'!A:A,'Budget 3 Juni 2024'!A448)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="449" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A449" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="B449" s="3"/>
-      <c r="C449" s="3"/>
-      <c r="D449" s="3"/>
-      <c r="E449" s="3"/>
-      <c r="F449" s="3"/>
-      <c r="G449" s="3"/>
-      <c r="H449" s="3"/>
+      <c r="B449" s="3">
+        <f>SUMIFS('II PD'!C:C,'II PD'!A:A,'Budget 3 Juni 2024'!A449)</f>
+        <v>0</v>
+      </c>
+      <c r="C449" s="3">
+        <f>SUMIFS('II PD'!D:D,'II PD'!A:A,'Budget 3 Juni 2024'!A449)</f>
+        <v>0</v>
+      </c>
+      <c r="D449" s="3">
+        <f>SUMIFS('II PD'!E:E,'II PD'!A:A,'Budget 3 Juni 2024'!A449)</f>
+        <v>0</v>
+      </c>
+      <c r="E449" s="3">
+        <f>SUMIFS('II PD'!F:F,'II PD'!A:A,'Budget 3 Juni 2024'!A449)</f>
+        <v>0</v>
+      </c>
+      <c r="F449" s="3">
+        <f>SUMIFS('II PD'!G:G,'II PD'!A:A,'Budget 3 Juni 2024'!A449)</f>
+        <v>0</v>
+      </c>
+      <c r="G449" s="3">
+        <f>SUMIFS('II PD'!H:H,'II PD'!A:A,'Budget 3 Juni 2024'!A449)</f>
+        <v>0</v>
+      </c>
+      <c r="H449" s="3">
+        <f>SUMIFS('II PD'!I:I,'II PD'!A:A,'Budget 3 Juni 2024'!A449)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="450" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A450" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="B450" s="3"/>
-      <c r="C450" s="3"/>
-      <c r="D450" s="3"/>
-      <c r="E450" s="3"/>
-      <c r="F450" s="3"/>
-      <c r="G450" s="3"/>
-      <c r="H450" s="3"/>
+      <c r="B450" s="3">
+        <f>SUMIFS('II PD'!C:C,'II PD'!A:A,'Budget 3 Juni 2024'!A450)</f>
+        <v>0</v>
+      </c>
+      <c r="C450" s="3">
+        <f>SUMIFS('II PD'!D:D,'II PD'!A:A,'Budget 3 Juni 2024'!A450)</f>
+        <v>0</v>
+      </c>
+      <c r="D450" s="3">
+        <f>SUMIFS('II PD'!E:E,'II PD'!A:A,'Budget 3 Juni 2024'!A450)</f>
+        <v>0</v>
+      </c>
+      <c r="E450" s="3">
+        <f>SUMIFS('II PD'!F:F,'II PD'!A:A,'Budget 3 Juni 2024'!A450)</f>
+        <v>0</v>
+      </c>
+      <c r="F450" s="3">
+        <f>SUMIFS('II PD'!G:G,'II PD'!A:A,'Budget 3 Juni 2024'!A450)</f>
+        <v>0</v>
+      </c>
+      <c r="G450" s="3">
+        <f>SUMIFS('II PD'!H:H,'II PD'!A:A,'Budget 3 Juni 2024'!A450)</f>
+        <v>0</v>
+      </c>
+      <c r="H450" s="3">
+        <f>SUMIFS('II PD'!I:I,'II PD'!A:A,'Budget 3 Juni 2024'!A450)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="451" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A451" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="B451" s="3"/>
-      <c r="C451" s="3"/>
-      <c r="D451" s="3"/>
-      <c r="E451" s="3"/>
-      <c r="F451" s="3"/>
-      <c r="G451" s="3"/>
-      <c r="H451" s="3"/>
+      <c r="B451" s="3">
+        <f>SUMIFS('II PD'!C:C,'II PD'!A:A,'Budget 3 Juni 2024'!A451)</f>
+        <v>0</v>
+      </c>
+      <c r="C451" s="3">
+        <f>SUMIFS('II PD'!D:D,'II PD'!A:A,'Budget 3 Juni 2024'!A451)</f>
+        <v>0</v>
+      </c>
+      <c r="D451" s="3">
+        <f>SUMIFS('II PD'!E:E,'II PD'!A:A,'Budget 3 Juni 2024'!A451)</f>
+        <v>0</v>
+      </c>
+      <c r="E451" s="3">
+        <f>SUMIFS('II PD'!F:F,'II PD'!A:A,'Budget 3 Juni 2024'!A451)</f>
+        <v>0</v>
+      </c>
+      <c r="F451" s="3">
+        <f>SUMIFS('II PD'!G:G,'II PD'!A:A,'Budget 3 Juni 2024'!A451)</f>
+        <v>0</v>
+      </c>
+      <c r="G451" s="3">
+        <f>SUMIFS('II PD'!H:H,'II PD'!A:A,'Budget 3 Juni 2024'!A451)</f>
+        <v>0</v>
+      </c>
+      <c r="H451" s="3">
+        <f>SUMIFS('II PD'!I:I,'II PD'!A:A,'Budget 3 Juni 2024'!A451)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="452" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A452" s="1" t="s">
         <v>130</v>
       </c>
       <c r="B452" s="3">
-        <v>372660000</v>
+        <f>SUMIFS('II PD'!C:C,'II PD'!A:A,'Budget 3 Juni 2024'!A452)</f>
+        <v>6000000</v>
       </c>
       <c r="C452" s="3">
-        <v>372660000</v>
+        <f>SUMIFS('II PD'!D:D,'II PD'!A:A,'Budget 3 Juni 2024'!A452)</f>
+        <v>1500000</v>
       </c>
       <c r="D452" s="3">
-        <v>8912700</v>
+        <f>SUMIFS('II PD'!E:E,'II PD'!A:A,'Budget 3 Juni 2024'!A452)</f>
+        <v>0</v>
       </c>
       <c r="E452" s="3">
-        <v>5604650</v>
+        <f>SUMIFS('II PD'!F:F,'II PD'!A:A,'Budget 3 Juni 2024'!A452)</f>
+        <v>0</v>
       </c>
       <c r="F452" s="3">
-        <v>14517350</v>
+        <f>SUMIFS('II PD'!G:G,'II PD'!A:A,'Budget 3 Juni 2024'!A452)</f>
+        <v>0</v>
       </c>
       <c r="G452" s="3">
-        <v>358142650</v>
+        <f>SUMIFS('II PD'!H:H,'II PD'!A:A,'Budget 3 Juni 2024'!A452)</f>
+        <v>1500000</v>
       </c>
       <c r="H452" s="3">
-        <v>0</v>
+        <f>SUMIFS('II PD'!I:I,'II PD'!A:A,'Budget 3 Juni 2024'!A452)</f>
+        <v>4500000</v>
       </c>
     </row>
     <row r="453" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A453" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="B453" s="3"/>
-      <c r="C453" s="3"/>
-      <c r="D453" s="3"/>
-      <c r="E453" s="3"/>
-      <c r="F453" s="3"/>
-      <c r="G453" s="3"/>
-      <c r="H453" s="3"/>
+      <c r="B453" s="3">
+        <f>SUMIFS('II PD'!C:C,'II PD'!A:A,'Budget 3 Juni 2024'!A453)</f>
+        <v>41000000</v>
+      </c>
+      <c r="C453" s="3">
+        <f>SUMIFS('II PD'!D:D,'II PD'!A:A,'Budget 3 Juni 2024'!A453)</f>
+        <v>10250000</v>
+      </c>
+      <c r="D453" s="3">
+        <f>SUMIFS('II PD'!E:E,'II PD'!A:A,'Budget 3 Juni 2024'!A453)</f>
+        <v>1997700</v>
+      </c>
+      <c r="E453" s="3">
+        <f>SUMIFS('II PD'!F:F,'II PD'!A:A,'Budget 3 Juni 2024'!A453)</f>
+        <v>998400</v>
+      </c>
+      <c r="F453" s="3">
+        <f>SUMIFS('II PD'!G:G,'II PD'!A:A,'Budget 3 Juni 2024'!A453)</f>
+        <v>2996100</v>
+      </c>
+      <c r="G453" s="3">
+        <f>SUMIFS('II PD'!H:H,'II PD'!A:A,'Budget 3 Juni 2024'!A453)</f>
+        <v>7253900</v>
+      </c>
+      <c r="H453" s="3">
+        <f>SUMIFS('II PD'!I:I,'II PD'!A:A,'Budget 3 Juni 2024'!A453)</f>
+        <v>30750000</v>
+      </c>
     </row>
     <row r="454" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A454" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="B454" s="3"/>
-      <c r="C454" s="3"/>
-      <c r="D454" s="3"/>
-      <c r="E454" s="3"/>
-      <c r="F454" s="3"/>
-      <c r="G454" s="3"/>
-      <c r="H454" s="3"/>
+      <c r="B454" s="3">
+        <f>SUMIFS('II PD'!C:C,'II PD'!A:A,'Budget 3 Juni 2024'!A454)</f>
+        <v>12000000</v>
+      </c>
+      <c r="C454" s="3">
+        <f>SUMIFS('II PD'!D:D,'II PD'!A:A,'Budget 3 Juni 2024'!A454)</f>
+        <v>3000000</v>
+      </c>
+      <c r="D454" s="3">
+        <f>SUMIFS('II PD'!E:E,'II PD'!A:A,'Budget 3 Juni 2024'!A454)</f>
+        <v>0</v>
+      </c>
+      <c r="E454" s="3">
+        <f>SUMIFS('II PD'!F:F,'II PD'!A:A,'Budget 3 Juni 2024'!A454)</f>
+        <v>0</v>
+      </c>
+      <c r="F454" s="3">
+        <f>SUMIFS('II PD'!G:G,'II PD'!A:A,'Budget 3 Juni 2024'!A454)</f>
+        <v>0</v>
+      </c>
+      <c r="G454" s="3">
+        <f>SUMIFS('II PD'!H:H,'II PD'!A:A,'Budget 3 Juni 2024'!A454)</f>
+        <v>3000000</v>
+      </c>
+      <c r="H454" s="3">
+        <f>SUMIFS('II PD'!I:I,'II PD'!A:A,'Budget 3 Juni 2024'!A454)</f>
+        <v>9000000</v>
+      </c>
     </row>
     <row r="455" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A455" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="B455" s="3"/>
-      <c r="C455" s="3"/>
-      <c r="D455" s="3"/>
-      <c r="E455" s="3"/>
-      <c r="F455" s="3"/>
-      <c r="G455" s="3"/>
-      <c r="H455" s="3"/>
+      <c r="B455" s="3">
+        <f>SUMIFS('II PD'!C:C,'II PD'!A:A,'Budget 3 Juni 2024'!A455)</f>
+        <v>171000000</v>
+      </c>
+      <c r="C455" s="3">
+        <f>SUMIFS('II PD'!D:D,'II PD'!A:A,'Budget 3 Juni 2024'!A455)</f>
+        <v>42750000</v>
+      </c>
+      <c r="D455" s="3">
+        <f>SUMIFS('II PD'!E:E,'II PD'!A:A,'Budget 3 Juni 2024'!A455)</f>
+        <v>5880000</v>
+      </c>
+      <c r="E455" s="3">
+        <f>SUMIFS('II PD'!F:F,'II PD'!A:A,'Budget 3 Juni 2024'!A455)</f>
+        <v>0</v>
+      </c>
+      <c r="F455" s="3">
+        <f>SUMIFS('II PD'!G:G,'II PD'!A:A,'Budget 3 Juni 2024'!A455)</f>
+        <v>5880000</v>
+      </c>
+      <c r="G455" s="3">
+        <f>SUMIFS('II PD'!H:H,'II PD'!A:A,'Budget 3 Juni 2024'!A455)</f>
+        <v>36870000</v>
+      </c>
+      <c r="H455" s="3">
+        <f>SUMIFS('II PD'!I:I,'II PD'!A:A,'Budget 3 Juni 2024'!A455)</f>
+        <v>128250000</v>
+      </c>
     </row>
     <row r="456" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A456" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="B456" s="3"/>
-      <c r="C456" s="3"/>
-      <c r="D456" s="3"/>
-      <c r="E456" s="3"/>
-      <c r="F456" s="3"/>
-      <c r="G456" s="3"/>
-      <c r="H456" s="3"/>
+      <c r="B456" s="3">
+        <f>SUMIFS('II PD'!C:C,'II PD'!A:A,'Budget 3 Juni 2024'!A456)</f>
+        <v>130000000</v>
+      </c>
+      <c r="C456" s="3">
+        <f>SUMIFS('II PD'!D:D,'II PD'!A:A,'Budget 3 Juni 2024'!A456)</f>
+        <v>32500000</v>
+      </c>
+      <c r="D456" s="3">
+        <f>SUMIFS('II PD'!E:E,'II PD'!A:A,'Budget 3 Juni 2024'!A456)</f>
+        <v>0</v>
+      </c>
+      <c r="E456" s="3">
+        <f>SUMIFS('II PD'!F:F,'II PD'!A:A,'Budget 3 Juni 2024'!A456)</f>
+        <v>7381250</v>
+      </c>
+      <c r="F456" s="3">
+        <f>SUMIFS('II PD'!G:G,'II PD'!A:A,'Budget 3 Juni 2024'!A456)</f>
+        <v>7381250</v>
+      </c>
+      <c r="G456" s="3">
+        <f>SUMIFS('II PD'!H:H,'II PD'!A:A,'Budget 3 Juni 2024'!A456)</f>
+        <v>25118750</v>
+      </c>
+      <c r="H456" s="3">
+        <f>SUMIFS('II PD'!I:I,'II PD'!A:A,'Budget 3 Juni 2024'!A456)</f>
+        <v>97500000</v>
+      </c>
     </row>
     <row r="457" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A457" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="B457" s="3"/>
-      <c r="C457" s="3"/>
-      <c r="D457" s="3"/>
-      <c r="E457" s="3"/>
-      <c r="F457" s="3"/>
-      <c r="G457" s="3"/>
-      <c r="H457" s="3"/>
+      <c r="B457" s="3">
+        <f>SUMIFS('II PD'!C:C,'II PD'!A:A,'Budget 3 Juni 2024'!A457)</f>
+        <v>6660000</v>
+      </c>
+      <c r="C457" s="3">
+        <f>SUMIFS('II PD'!D:D,'II PD'!A:A,'Budget 3 Juni 2024'!A457)</f>
+        <v>1665000</v>
+      </c>
+      <c r="D457" s="3">
+        <f>SUMIFS('II PD'!E:E,'II PD'!A:A,'Budget 3 Juni 2024'!A457)</f>
+        <v>1665000</v>
+      </c>
+      <c r="E457" s="3">
+        <f>SUMIFS('II PD'!F:F,'II PD'!A:A,'Budget 3 Juni 2024'!A457)</f>
+        <v>0</v>
+      </c>
+      <c r="F457" s="3">
+        <f>SUMIFS('II PD'!G:G,'II PD'!A:A,'Budget 3 Juni 2024'!A457)</f>
+        <v>1665000</v>
+      </c>
+      <c r="G457" s="3">
+        <f>SUMIFS('II PD'!H:H,'II PD'!A:A,'Budget 3 Juni 2024'!A457)</f>
+        <v>0</v>
+      </c>
+      <c r="H457" s="3">
+        <f>SUMIFS('II PD'!I:I,'II PD'!A:A,'Budget 3 Juni 2024'!A457)</f>
+        <v>4995000</v>
+      </c>
     </row>
     <row r="458" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A458" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="B458" s="3"/>
-      <c r="C458" s="3"/>
-      <c r="D458" s="3"/>
-      <c r="E458" s="3"/>
-      <c r="F458" s="3"/>
-      <c r="G458" s="3"/>
-      <c r="H458" s="3"/>
+      <c r="B458" s="3">
+        <f>SUMIFS('II PD'!C:C,'II PD'!A:A,'Budget 3 Juni 2024'!A458)</f>
+        <v>6000000</v>
+      </c>
+      <c r="C458" s="3">
+        <f>SUMIFS('II PD'!D:D,'II PD'!A:A,'Budget 3 Juni 2024'!A458)</f>
+        <v>1500000</v>
+      </c>
+      <c r="D458" s="3">
+        <f>SUMIFS('II PD'!E:E,'II PD'!A:A,'Budget 3 Juni 2024'!A458)</f>
+        <v>0</v>
+      </c>
+      <c r="E458" s="3">
+        <f>SUMIFS('II PD'!F:F,'II PD'!A:A,'Budget 3 Juni 2024'!A458)</f>
+        <v>0</v>
+      </c>
+      <c r="F458" s="3">
+        <f>SUMIFS('II PD'!G:G,'II PD'!A:A,'Budget 3 Juni 2024'!A458)</f>
+        <v>0</v>
+      </c>
+      <c r="G458" s="3">
+        <f>SUMIFS('II PD'!H:H,'II PD'!A:A,'Budget 3 Juni 2024'!A458)</f>
+        <v>1500000</v>
+      </c>
+      <c r="H458" s="3">
+        <f>SUMIFS('II PD'!I:I,'II PD'!A:A,'Budget 3 Juni 2024'!A458)</f>
+        <v>4500000</v>
+      </c>
     </row>
     <row r="459" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A459" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="B459" s="3"/>
-      <c r="C459" s="3"/>
-      <c r="D459" s="3"/>
-      <c r="E459" s="3"/>
-      <c r="F459" s="3"/>
-      <c r="G459" s="3"/>
-      <c r="H459" s="3"/>
+      <c r="B459" s="3">
+        <f>SUMIFS('II PD'!C:C,'II PD'!A:A,'Budget 3 Juni 2024'!A459)</f>
+        <v>0</v>
+      </c>
+      <c r="C459" s="3">
+        <f>SUMIFS('II PD'!D:D,'II PD'!A:A,'Budget 3 Juni 2024'!A459)</f>
+        <v>0</v>
+      </c>
+      <c r="D459" s="3">
+        <f>SUMIFS('II PD'!E:E,'II PD'!A:A,'Budget 3 Juni 2024'!A459)</f>
+        <v>0</v>
+      </c>
+      <c r="E459" s="3">
+        <f>SUMIFS('II PD'!F:F,'II PD'!A:A,'Budget 3 Juni 2024'!A459)</f>
+        <v>0</v>
+      </c>
+      <c r="F459" s="3">
+        <f>SUMIFS('II PD'!G:G,'II PD'!A:A,'Budget 3 Juni 2024'!A459)</f>
+        <v>0</v>
+      </c>
+      <c r="G459" s="3">
+        <f>SUMIFS('II PD'!H:H,'II PD'!A:A,'Budget 3 Juni 2024'!A459)</f>
+        <v>0</v>
+      </c>
+      <c r="H459" s="3">
+        <f>SUMIFS('II PD'!I:I,'II PD'!A:A,'Budget 3 Juni 2024'!A459)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="460" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A460" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="B460" s="3"/>
-      <c r="C460" s="3"/>
-      <c r="D460" s="3"/>
-      <c r="E460" s="3"/>
-      <c r="F460" s="3"/>
-      <c r="G460" s="3"/>
-      <c r="H460" s="3"/>
+      <c r="B460" s="3">
+        <f>SUMIFS('II PD'!C:C,'II PD'!A:A,'Budget 3 Juni 2024'!A460)</f>
+        <v>0</v>
+      </c>
+      <c r="C460" s="3">
+        <f>SUMIFS('II PD'!D:D,'II PD'!A:A,'Budget 3 Juni 2024'!A460)</f>
+        <v>0</v>
+      </c>
+      <c r="D460" s="3">
+        <f>SUMIFS('II PD'!E:E,'II PD'!A:A,'Budget 3 Juni 2024'!A460)</f>
+        <v>0</v>
+      </c>
+      <c r="E460" s="3">
+        <f>SUMIFS('II PD'!F:F,'II PD'!A:A,'Budget 3 Juni 2024'!A460)</f>
+        <v>0</v>
+      </c>
+      <c r="F460" s="3">
+        <f>SUMIFS('II PD'!G:G,'II PD'!A:A,'Budget 3 Juni 2024'!A460)</f>
+        <v>0</v>
+      </c>
+      <c r="G460" s="3">
+        <f>SUMIFS('II PD'!H:H,'II PD'!A:A,'Budget 3 Juni 2024'!A460)</f>
+        <v>0</v>
+      </c>
+      <c r="H460" s="3">
+        <f>SUMIFS('II PD'!I:I,'II PD'!A:A,'Budget 3 Juni 2024'!A460)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="461" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A461" s="1" t="s">
         <v>139</v>
       </c>
-      <c r="B461" s="3"/>
-      <c r="C461" s="3"/>
-      <c r="D461" s="3"/>
-      <c r="E461" s="3"/>
-      <c r="F461" s="3"/>
-      <c r="G461" s="3"/>
-      <c r="H461" s="3"/>
+      <c r="B461" s="3">
+        <f>SUMIFS('II PD'!C:C,'II PD'!A:A,'Budget 3 Juni 2024'!A461)</f>
+        <v>0</v>
+      </c>
+      <c r="C461" s="3">
+        <f>SUMIFS('II PD'!D:D,'II PD'!A:A,'Budget 3 Juni 2024'!A461)</f>
+        <v>0</v>
+      </c>
+      <c r="D461" s="3">
+        <f>SUMIFS('II PD'!E:E,'II PD'!A:A,'Budget 3 Juni 2024'!A461)</f>
+        <v>0</v>
+      </c>
+      <c r="E461" s="3">
+        <f>SUMIFS('II PD'!F:F,'II PD'!A:A,'Budget 3 Juni 2024'!A461)</f>
+        <v>0</v>
+      </c>
+      <c r="F461" s="3">
+        <f>SUMIFS('II PD'!G:G,'II PD'!A:A,'Budget 3 Juni 2024'!A461)</f>
+        <v>0</v>
+      </c>
+      <c r="G461" s="3">
+        <f>SUMIFS('II PD'!H:H,'II PD'!A:A,'Budget 3 Juni 2024'!A461)</f>
+        <v>0</v>
+      </c>
+      <c r="H461" s="3">
+        <f>SUMIFS('II PD'!I:I,'II PD'!A:A,'Budget 3 Juni 2024'!A461)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="462" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A462" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="B462" s="3"/>
-      <c r="C462" s="3"/>
-      <c r="D462" s="3"/>
-      <c r="E462" s="3"/>
-      <c r="F462" s="3"/>
-      <c r="G462" s="3"/>
-      <c r="H462" s="3"/>
+      <c r="B462" s="3">
+        <f>SUMIFS('II PD'!C:C,'II PD'!A:A,'Budget 3 Juni 2024'!A462)</f>
+        <v>0</v>
+      </c>
+      <c r="C462" s="3">
+        <f>SUMIFS('II PD'!D:D,'II PD'!A:A,'Budget 3 Juni 2024'!A462)</f>
+        <v>0</v>
+      </c>
+      <c r="D462" s="3">
+        <f>SUMIFS('II PD'!E:E,'II PD'!A:A,'Budget 3 Juni 2024'!A462)</f>
+        <v>0</v>
+      </c>
+      <c r="E462" s="3">
+        <f>SUMIFS('II PD'!F:F,'II PD'!A:A,'Budget 3 Juni 2024'!A462)</f>
+        <v>0</v>
+      </c>
+      <c r="F462" s="3">
+        <f>SUMIFS('II PD'!G:G,'II PD'!A:A,'Budget 3 Juni 2024'!A462)</f>
+        <v>0</v>
+      </c>
+      <c r="G462" s="3">
+        <f>SUMIFS('II PD'!H:H,'II PD'!A:A,'Budget 3 Juni 2024'!A462)</f>
+        <v>0</v>
+      </c>
+      <c r="H462" s="3">
+        <f>SUMIFS('II PD'!I:I,'II PD'!A:A,'Budget 3 Juni 2024'!A462)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="463" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A463" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="B463" s="3"/>
-      <c r="C463" s="3"/>
-      <c r="D463" s="3"/>
-      <c r="E463" s="3"/>
-      <c r="F463" s="3"/>
-      <c r="G463" s="3"/>
-      <c r="H463" s="3"/>
+      <c r="B463" s="3">
+        <f>SUMIFS('II PD'!C:C,'II PD'!A:A,'Budget 3 Juni 2024'!A463)</f>
+        <v>0</v>
+      </c>
+      <c r="C463" s="3">
+        <f>SUMIFS('II PD'!D:D,'II PD'!A:A,'Budget 3 Juni 2024'!A463)</f>
+        <v>0</v>
+      </c>
+      <c r="D463" s="3">
+        <f>SUMIFS('II PD'!E:E,'II PD'!A:A,'Budget 3 Juni 2024'!A463)</f>
+        <v>0</v>
+      </c>
+      <c r="E463" s="3">
+        <f>SUMIFS('II PD'!F:F,'II PD'!A:A,'Budget 3 Juni 2024'!A463)</f>
+        <v>0</v>
+      </c>
+      <c r="F463" s="3">
+        <f>SUMIFS('II PD'!G:G,'II PD'!A:A,'Budget 3 Juni 2024'!A463)</f>
+        <v>0</v>
+      </c>
+      <c r="G463" s="3">
+        <f>SUMIFS('II PD'!H:H,'II PD'!A:A,'Budget 3 Juni 2024'!A463)</f>
+        <v>0</v>
+      </c>
+      <c r="H463" s="3">
+        <f>SUMIFS('II PD'!I:I,'II PD'!A:A,'Budget 3 Juni 2024'!A463)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="464" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A464" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="B464" s="3"/>
-      <c r="C464" s="3"/>
-      <c r="D464" s="3"/>
-      <c r="E464" s="3"/>
-      <c r="F464" s="3"/>
-      <c r="G464" s="3"/>
-      <c r="H464" s="3"/>
+      <c r="B464" s="3">
+        <f>SUMIFS('II PD'!C:C,'II PD'!A:A,'Budget 3 Juni 2024'!A464)</f>
+        <v>0</v>
+      </c>
+      <c r="C464" s="3">
+        <f>SUMIFS('II PD'!D:D,'II PD'!A:A,'Budget 3 Juni 2024'!A464)</f>
+        <v>0</v>
+      </c>
+      <c r="D464" s="3">
+        <f>SUMIFS('II PD'!E:E,'II PD'!A:A,'Budget 3 Juni 2024'!A464)</f>
+        <v>0</v>
+      </c>
+      <c r="E464" s="3">
+        <f>SUMIFS('II PD'!F:F,'II PD'!A:A,'Budget 3 Juni 2024'!A464)</f>
+        <v>0</v>
+      </c>
+      <c r="F464" s="3">
+        <f>SUMIFS('II PD'!G:G,'II PD'!A:A,'Budget 3 Juni 2024'!A464)</f>
+        <v>0</v>
+      </c>
+      <c r="G464" s="3">
+        <f>SUMIFS('II PD'!H:H,'II PD'!A:A,'Budget 3 Juni 2024'!A464)</f>
+        <v>0</v>
+      </c>
+      <c r="H464" s="3">
+        <f>SUMIFS('II PD'!I:I,'II PD'!A:A,'Budget 3 Juni 2024'!A464)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="465" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A465" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="B465" s="3"/>
-      <c r="C465" s="3"/>
-      <c r="D465" s="3"/>
-      <c r="E465" s="3"/>
-      <c r="F465" s="3"/>
-      <c r="G465" s="3"/>
-      <c r="H465" s="3"/>
+      <c r="B465" s="3">
+        <f>SUMIFS('II PD'!C:C,'II PD'!A:A,'Budget 3 Juni 2024'!A465)</f>
+        <v>0</v>
+      </c>
+      <c r="C465" s="3">
+        <f>SUMIFS('II PD'!D:D,'II PD'!A:A,'Budget 3 Juni 2024'!A465)</f>
+        <v>0</v>
+      </c>
+      <c r="D465" s="3">
+        <f>SUMIFS('II PD'!E:E,'II PD'!A:A,'Budget 3 Juni 2024'!A465)</f>
+        <v>0</v>
+      </c>
+      <c r="E465" s="3">
+        <f>SUMIFS('II PD'!F:F,'II PD'!A:A,'Budget 3 Juni 2024'!A465)</f>
+        <v>0</v>
+      </c>
+      <c r="F465" s="3">
+        <f>SUMIFS('II PD'!G:G,'II PD'!A:A,'Budget 3 Juni 2024'!A465)</f>
+        <v>0</v>
+      </c>
+      <c r="G465" s="3">
+        <f>SUMIFS('II PD'!H:H,'II PD'!A:A,'Budget 3 Juni 2024'!A465)</f>
+        <v>0</v>
+      </c>
+      <c r="H465" s="3">
+        <f>SUMIFS('II PD'!I:I,'II PD'!A:A,'Budget 3 Juni 2024'!A465)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="466" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A466" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="B466" s="3"/>
-      <c r="C466" s="3"/>
-      <c r="D466" s="3"/>
-      <c r="E466" s="3"/>
-      <c r="F466" s="3"/>
-      <c r="G466" s="3"/>
-      <c r="H466" s="3"/>
+      <c r="B466" s="3">
+        <f>SUMIFS('II PD'!C:C,'II PD'!A:A,'Budget 3 Juni 2024'!A466)</f>
+        <v>0</v>
+      </c>
+      <c r="C466" s="3">
+        <f>SUMIFS('II PD'!D:D,'II PD'!A:A,'Budget 3 Juni 2024'!A466)</f>
+        <v>0</v>
+      </c>
+      <c r="D466" s="3">
+        <f>SUMIFS('II PD'!E:E,'II PD'!A:A,'Budget 3 Juni 2024'!A466)</f>
+        <v>0</v>
+      </c>
+      <c r="E466" s="3">
+        <f>SUMIFS('II PD'!F:F,'II PD'!A:A,'Budget 3 Juni 2024'!A466)</f>
+        <v>0</v>
+      </c>
+      <c r="F466" s="3">
+        <f>SUMIFS('II PD'!G:G,'II PD'!A:A,'Budget 3 Juni 2024'!A466)</f>
+        <v>0</v>
+      </c>
+      <c r="G466" s="3">
+        <f>SUMIFS('II PD'!H:H,'II PD'!A:A,'Budget 3 Juni 2024'!A466)</f>
+        <v>0</v>
+      </c>
+      <c r="H466" s="3">
+        <f>SUMIFS('II PD'!I:I,'II PD'!A:A,'Budget 3 Juni 2024'!A466)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="467" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A467" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="B467" s="3"/>
-      <c r="C467" s="3"/>
-      <c r="D467" s="3"/>
-      <c r="E467" s="3"/>
-      <c r="F467" s="3"/>
-      <c r="G467" s="3"/>
-      <c r="H467" s="3"/>
+      <c r="B467" s="3">
+        <f>SUMIFS('II PD'!C:C,'II PD'!A:A,'Budget 3 Juni 2024'!A467)</f>
+        <v>0</v>
+      </c>
+      <c r="C467" s="3">
+        <f>SUMIFS('II PD'!D:D,'II PD'!A:A,'Budget 3 Juni 2024'!A467)</f>
+        <v>0</v>
+      </c>
+      <c r="D467" s="3">
+        <f>SUMIFS('II PD'!E:E,'II PD'!A:A,'Budget 3 Juni 2024'!A467)</f>
+        <v>0</v>
+      </c>
+      <c r="E467" s="3">
+        <f>SUMIFS('II PD'!F:F,'II PD'!A:A,'Budget 3 Juni 2024'!A467)</f>
+        <v>0</v>
+      </c>
+      <c r="F467" s="3">
+        <f>SUMIFS('II PD'!G:G,'II PD'!A:A,'Budget 3 Juni 2024'!A467)</f>
+        <v>0</v>
+      </c>
+      <c r="G467" s="3">
+        <f>SUMIFS('II PD'!H:H,'II PD'!A:A,'Budget 3 Juni 2024'!A467)</f>
+        <v>0</v>
+      </c>
+      <c r="H467" s="3">
+        <f>SUMIFS('II PD'!I:I,'II PD'!A:A,'Budget 3 Juni 2024'!A467)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="468" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A468" s="1" t="s">
         <v>146</v>
       </c>
-      <c r="B468" s="3"/>
-      <c r="C468" s="3"/>
-      <c r="D468" s="3"/>
-      <c r="E468" s="3"/>
-      <c r="F468" s="3"/>
-      <c r="G468" s="3"/>
-      <c r="H468" s="3"/>
+      <c r="B468" s="3">
+        <f>SUMIFS('II PD'!C:C,'II PD'!A:A,'Budget 3 Juni 2024'!A468)</f>
+        <v>0</v>
+      </c>
+      <c r="C468" s="3">
+        <f>SUMIFS('II PD'!D:D,'II PD'!A:A,'Budget 3 Juni 2024'!A468)</f>
+        <v>0</v>
+      </c>
+      <c r="D468" s="3">
+        <f>SUMIFS('II PD'!E:E,'II PD'!A:A,'Budget 3 Juni 2024'!A468)</f>
+        <v>0</v>
+      </c>
+      <c r="E468" s="3">
+        <f>SUMIFS('II PD'!F:F,'II PD'!A:A,'Budget 3 Juni 2024'!A468)</f>
+        <v>0</v>
+      </c>
+      <c r="F468" s="3">
+        <f>SUMIFS('II PD'!G:G,'II PD'!A:A,'Budget 3 Juni 2024'!A468)</f>
+        <v>0</v>
+      </c>
+      <c r="G468" s="3">
+        <f>SUMIFS('II PD'!H:H,'II PD'!A:A,'Budget 3 Juni 2024'!A468)</f>
+        <v>0</v>
+      </c>
+      <c r="H468" s="3">
+        <f>SUMIFS('II PD'!I:I,'II PD'!A:A,'Budget 3 Juni 2024'!A468)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="469" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A469" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="B469" s="3"/>
-      <c r="C469" s="3"/>
-      <c r="D469" s="3"/>
-      <c r="E469" s="3"/>
-      <c r="F469" s="3"/>
-      <c r="G469" s="3"/>
-      <c r="H469" s="3"/>
+      <c r="B469" s="3">
+        <f>SUMIFS('II PD'!C:C,'II PD'!A:A,'Budget 3 Juni 2024'!A469)</f>
+        <v>0</v>
+      </c>
+      <c r="C469" s="3">
+        <f>SUMIFS('II PD'!D:D,'II PD'!A:A,'Budget 3 Juni 2024'!A469)</f>
+        <v>0</v>
+      </c>
+      <c r="D469" s="3">
+        <f>SUMIFS('II PD'!E:E,'II PD'!A:A,'Budget 3 Juni 2024'!A469)</f>
+        <v>0</v>
+      </c>
+      <c r="E469" s="3">
+        <f>SUMIFS('II PD'!F:F,'II PD'!A:A,'Budget 3 Juni 2024'!A469)</f>
+        <v>0</v>
+      </c>
+      <c r="F469" s="3">
+        <f>SUMIFS('II PD'!G:G,'II PD'!A:A,'Budget 3 Juni 2024'!A469)</f>
+        <v>0</v>
+      </c>
+      <c r="G469" s="3">
+        <f>SUMIFS('II PD'!H:H,'II PD'!A:A,'Budget 3 Juni 2024'!A469)</f>
+        <v>0</v>
+      </c>
+      <c r="H469" s="3">
+        <f>SUMIFS('II PD'!I:I,'II PD'!A:A,'Budget 3 Juni 2024'!A469)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="470" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A470" s="1" t="s">
         <v>148</v>
       </c>
-      <c r="B470" s="3"/>
-      <c r="C470" s="3"/>
-      <c r="D470" s="3"/>
-      <c r="E470" s="3"/>
-      <c r="F470" s="3"/>
-      <c r="G470" s="3"/>
-      <c r="H470" s="3"/>
+      <c r="B470" s="3">
+        <f>SUMIFS('II PD'!C:C,'II PD'!A:A,'Budget 3 Juni 2024'!A470)</f>
+        <v>0</v>
+      </c>
+      <c r="C470" s="3">
+        <f>SUMIFS('II PD'!D:D,'II PD'!A:A,'Budget 3 Juni 2024'!A470)</f>
+        <v>0</v>
+      </c>
+      <c r="D470" s="3">
+        <f>SUMIFS('II PD'!E:E,'II PD'!A:A,'Budget 3 Juni 2024'!A470)</f>
+        <v>0</v>
+      </c>
+      <c r="E470" s="3">
+        <f>SUMIFS('II PD'!F:F,'II PD'!A:A,'Budget 3 Juni 2024'!A470)</f>
+        <v>0</v>
+      </c>
+      <c r="F470" s="3">
+        <f>SUMIFS('II PD'!G:G,'II PD'!A:A,'Budget 3 Juni 2024'!A470)</f>
+        <v>0</v>
+      </c>
+      <c r="G470" s="3">
+        <f>SUMIFS('II PD'!H:H,'II PD'!A:A,'Budget 3 Juni 2024'!A470)</f>
+        <v>0</v>
+      </c>
+      <c r="H470" s="3">
+        <f>SUMIFS('II PD'!I:I,'II PD'!A:A,'Budget 3 Juni 2024'!A470)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="471" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A471" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="B471" s="3"/>
-      <c r="C471" s="3"/>
-      <c r="D471" s="3"/>
-      <c r="E471" s="3"/>
-      <c r="F471" s="3"/>
-      <c r="G471" s="3"/>
-      <c r="H471" s="3"/>
+      <c r="B471" s="3">
+        <f>SUMIFS('II PD'!C:C,'II PD'!A:A,'Budget 3 Juni 2024'!A471)</f>
+        <v>0</v>
+      </c>
+      <c r="C471" s="3">
+        <f>SUMIFS('II PD'!D:D,'II PD'!A:A,'Budget 3 Juni 2024'!A471)</f>
+        <v>0</v>
+      </c>
+      <c r="D471" s="3">
+        <f>SUMIFS('II PD'!E:E,'II PD'!A:A,'Budget 3 Juni 2024'!A471)</f>
+        <v>0</v>
+      </c>
+      <c r="E471" s="3">
+        <f>SUMIFS('II PD'!F:F,'II PD'!A:A,'Budget 3 Juni 2024'!A471)</f>
+        <v>0</v>
+      </c>
+      <c r="F471" s="3">
+        <f>SUMIFS('II PD'!G:G,'II PD'!A:A,'Budget 3 Juni 2024'!A471)</f>
+        <v>0</v>
+      </c>
+      <c r="G471" s="3">
+        <f>SUMIFS('II PD'!H:H,'II PD'!A:A,'Budget 3 Juni 2024'!A471)</f>
+        <v>0</v>
+      </c>
+      <c r="H471" s="3">
+        <f>SUMIFS('II PD'!I:I,'II PD'!A:A,'Budget 3 Juni 2024'!A471)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="472" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A472" s="1" t="s">
         <v>150</v>
       </c>
       <c r="B472" s="3">
-        <v>2349760730</v>
+        <f>SUMIFS('II PD'!C:C,'II PD'!A:A,'Budget 3 Juni 2024'!A472)</f>
+        <v>2349761000</v>
       </c>
       <c r="C472" s="3">
-        <v>2349760730</v>
+        <f>SUMIFS('II PD'!D:D,'II PD'!A:A,'Budget 3 Juni 2024'!A472)</f>
+        <v>1085685500</v>
       </c>
       <c r="D472" s="3">
-        <v>429270952</v>
+        <f>SUMIFS('II PD'!E:E,'II PD'!A:A,'Budget 3 Juni 2024'!A472)</f>
+        <v>443295900</v>
       </c>
       <c r="E472" s="3">
-        <v>90620828</v>
+        <f>SUMIFS('II PD'!F:F,'II PD'!A:A,'Budget 3 Juni 2024'!A472)</f>
+        <v>80000880</v>
       </c>
       <c r="F472" s="3">
-        <v>519891780</v>
+        <f>SUMIFS('II PD'!G:G,'II PD'!A:A,'Budget 3 Juni 2024'!A472)</f>
+        <v>523296780</v>
       </c>
       <c r="G472" s="3">
-        <v>1829868950</v>
+        <f>SUMIFS('II PD'!H:H,'II PD'!A:A,'Budget 3 Juni 2024'!A472)</f>
+        <v>562388720</v>
       </c>
       <c r="H472" s="3">
-        <v>0</v>
+        <f>SUMIFS('II PD'!I:I,'II PD'!A:A,'Budget 3 Juni 2024'!A472)</f>
+        <v>1264075500</v>
       </c>
     </row>
     <row r="473" spans="1:8" x14ac:dyDescent="0.45">
@@ -14891,4 +15977,1489 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{74037102-CAE5-4DA3-AC4F-276E222EA2EC}">
+  <dimension ref="A1:I54"/>
+  <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.25" customHeight="1" zeroHeight="1" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="1" max="1" width="60.86328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="5" width="15.265625" style="12" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.265625" style="12" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="15.265625" style="12" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.265625" style="12" bestFit="1" customWidth="1"/>
+    <col min="10" max="16384" width="9" hidden="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>151</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="I1" s="8" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A2" t="s">
+        <v>98</v>
+      </c>
+      <c r="B2" s="4">
+        <v>873740000</v>
+      </c>
+      <c r="C2" s="5">
+        <f>B2</f>
+        <v>873740000</v>
+      </c>
+      <c r="D2" s="5">
+        <f>C2/2</f>
+        <v>436870000</v>
+      </c>
+      <c r="E2" s="4">
+        <f>IF(B2="","",G2-F2)</f>
+        <v>404360000</v>
+      </c>
+      <c r="F2" s="5">
+        <v>35605052</v>
+      </c>
+      <c r="G2" s="5">
+        <v>439965052</v>
+      </c>
+      <c r="H2" s="4">
+        <f>IF(B2="","",D2-G2)</f>
+        <v>-3095052</v>
+      </c>
+      <c r="I2" s="4">
+        <f>IF(B2="","",C2-D2)</f>
+        <v>436870000</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+      <c r="A3" t="s">
+        <v>99</v>
+      </c>
+      <c r="B3" s="4"/>
+      <c r="C3" s="5">
+        <f t="shared" ref="C3:C27" si="0">B3</f>
+        <v>0</v>
+      </c>
+      <c r="D3" s="5">
+        <f t="shared" ref="D3:D27" si="1">C3/2</f>
+        <v>0</v>
+      </c>
+      <c r="E3" s="4" t="str">
+        <f t="shared" ref="E3:E53" si="2">IF(B3="","",G3-F3)</f>
+        <v/>
+      </c>
+      <c r="F3" s="5"/>
+      <c r="G3" s="5"/>
+      <c r="H3" s="4" t="str">
+        <f t="shared" ref="H3:H53" si="3">IF(B3="","",D3-G3)</f>
+        <v/>
+      </c>
+      <c r="I3" s="4" t="str">
+        <f t="shared" ref="I3:I53" si="4">IF(B3="","",C3-D3)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+      <c r="A4" t="s">
+        <v>100</v>
+      </c>
+      <c r="B4" s="4"/>
+      <c r="C4" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="D4" s="5">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="E4" s="4" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F4" s="5"/>
+      <c r="G4" s="5"/>
+      <c r="H4" s="4" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="I4" s="4" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="5" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+      <c r="A5" t="s">
+        <v>101</v>
+      </c>
+      <c r="B5" s="4"/>
+      <c r="C5" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="D5" s="5">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="E5" s="4" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F5" s="5"/>
+      <c r="G5" s="5"/>
+      <c r="H5" s="4" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="I5" s="4" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="6" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+      <c r="A6" t="s">
+        <v>102</v>
+      </c>
+      <c r="B6" s="4"/>
+      <c r="C6" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="D6" s="5">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="E6" s="4" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F6" s="5"/>
+      <c r="G6" s="5"/>
+      <c r="H6" s="4" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="I6" s="4" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="7" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+      <c r="A7" t="s">
+        <v>103</v>
+      </c>
+      <c r="B7" s="4"/>
+      <c r="C7" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="D7" s="5">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="E7" s="4" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F7" s="5"/>
+      <c r="G7" s="5"/>
+      <c r="H7" s="4" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="I7" s="4" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="8" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+      <c r="A8" t="s">
+        <v>104</v>
+      </c>
+      <c r="B8" s="4"/>
+      <c r="C8" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="D8" s="5">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="E8" s="4" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F8" s="5"/>
+      <c r="G8" s="5"/>
+      <c r="H8" s="4" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="I8" s="4" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="9" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+      <c r="A9" t="s">
+        <v>105</v>
+      </c>
+      <c r="B9" s="4"/>
+      <c r="C9" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="D9" s="5">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="E9" s="4" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F9" s="5"/>
+      <c r="G9" s="5"/>
+      <c r="H9" s="4" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="I9" s="4" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="10" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+      <c r="A10" t="s">
+        <v>106</v>
+      </c>
+      <c r="B10" s="4"/>
+      <c r="C10" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="D10" s="5">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="E10" s="4" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F10" s="5"/>
+      <c r="G10" s="5"/>
+      <c r="H10" s="4" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="I10" s="4" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="11" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+      <c r="A11" t="s">
+        <v>107</v>
+      </c>
+      <c r="B11" s="4"/>
+      <c r="C11" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="D11" s="5">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="E11" s="4" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F11" s="5"/>
+      <c r="G11" s="5"/>
+      <c r="H11" s="4" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="I11" s="4" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="12" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+      <c r="A12" t="s">
+        <v>108</v>
+      </c>
+      <c r="B12" s="4"/>
+      <c r="C12" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="D12" s="5">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="E12" s="4" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F12" s="5"/>
+      <c r="G12" s="5"/>
+      <c r="H12" s="4" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="I12" s="4" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="13" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+      <c r="A13" t="s">
+        <v>109</v>
+      </c>
+      <c r="B13" s="4"/>
+      <c r="C13" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="D13" s="5">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="E13" s="4" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F13" s="5"/>
+      <c r="G13" s="5"/>
+      <c r="H13" s="4" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="I13" s="4" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="14" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+      <c r="A14" t="s">
+        <v>110</v>
+      </c>
+      <c r="B14" s="4"/>
+      <c r="C14" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="D14" s="5">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="E14" s="4" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F14" s="5"/>
+      <c r="G14" s="5"/>
+      <c r="H14" s="4" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="I14" s="4" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="15" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+      <c r="A15" t="s">
+        <v>111</v>
+      </c>
+      <c r="B15" s="4"/>
+      <c r="C15" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="D15" s="5">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="E15" s="4" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F15" s="5"/>
+      <c r="G15" s="5"/>
+      <c r="H15" s="4" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="I15" s="4" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="16" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+      <c r="A16" t="s">
+        <v>112</v>
+      </c>
+      <c r="B16" s="4"/>
+      <c r="C16" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="D16" s="5">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="E16" s="4" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F16" s="5"/>
+      <c r="G16" s="5"/>
+      <c r="H16" s="4" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="I16" s="4" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="17" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+      <c r="A17" t="s">
+        <v>113</v>
+      </c>
+      <c r="B17" s="4"/>
+      <c r="C17" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="D17" s="5">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="E17" s="4" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F17" s="5"/>
+      <c r="G17" s="5"/>
+      <c r="H17" s="4" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="I17" s="4" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="18" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+      <c r="A18" t="s">
+        <v>114</v>
+      </c>
+      <c r="B18" s="4"/>
+      <c r="C18" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="D18" s="5">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="E18" s="4" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F18" s="5"/>
+      <c r="G18" s="5"/>
+      <c r="H18" s="4" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="I18" s="4" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A19" t="s">
+        <v>115</v>
+      </c>
+      <c r="B19" s="4">
+        <v>474786000</v>
+      </c>
+      <c r="C19" s="5">
+        <f t="shared" si="0"/>
+        <v>474786000</v>
+      </c>
+      <c r="D19" s="5">
+        <f t="shared" si="1"/>
+        <v>237393000</v>
+      </c>
+      <c r="E19" s="4">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="F19" s="5"/>
+      <c r="G19" s="5"/>
+      <c r="H19" s="4">
+        <f t="shared" si="3"/>
+        <v>237393000</v>
+      </c>
+      <c r="I19" s="4">
+        <f t="shared" si="4"/>
+        <v>237393000</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A20" t="s">
+        <v>116</v>
+      </c>
+      <c r="B20" s="4">
+        <v>208425000</v>
+      </c>
+      <c r="C20" s="5">
+        <f t="shared" si="0"/>
+        <v>208425000</v>
+      </c>
+      <c r="D20" s="5">
+        <f t="shared" si="1"/>
+        <v>104212500</v>
+      </c>
+      <c r="E20" s="4">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="F20" s="5"/>
+      <c r="G20" s="5"/>
+      <c r="H20" s="4">
+        <f t="shared" si="3"/>
+        <v>104212500</v>
+      </c>
+      <c r="I20" s="4">
+        <f t="shared" si="4"/>
+        <v>104212500</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A21" t="s">
+        <v>117</v>
+      </c>
+      <c r="B21" s="4">
+        <v>20000000</v>
+      </c>
+      <c r="C21" s="5">
+        <f>B21</f>
+        <v>20000000</v>
+      </c>
+      <c r="D21" s="5">
+        <v>13970000</v>
+      </c>
+      <c r="E21" s="4">
+        <f t="shared" si="2"/>
+        <v>13970000</v>
+      </c>
+      <c r="F21" s="5"/>
+      <c r="G21" s="5">
+        <v>13970000</v>
+      </c>
+      <c r="H21" s="4">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="I21" s="4">
+        <f t="shared" si="4"/>
+        <v>6030000</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A22" t="s">
+        <v>118</v>
+      </c>
+      <c r="B22" s="4">
+        <v>220000000</v>
+      </c>
+      <c r="C22" s="5">
+        <f t="shared" si="0"/>
+        <v>220000000</v>
+      </c>
+      <c r="D22" s="5">
+        <f t="shared" si="1"/>
+        <v>110000000</v>
+      </c>
+      <c r="E22" s="4">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="F22" s="5">
+        <v>29896778</v>
+      </c>
+      <c r="G22" s="5">
+        <v>29896778</v>
+      </c>
+      <c r="H22" s="4">
+        <f t="shared" si="3"/>
+        <v>80103222</v>
+      </c>
+      <c r="I22" s="4">
+        <f t="shared" si="4"/>
+        <v>110000000</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A23" t="s">
+        <v>119</v>
+      </c>
+      <c r="B23" s="4">
+        <v>75000000</v>
+      </c>
+      <c r="C23" s="5">
+        <f t="shared" si="0"/>
+        <v>75000000</v>
+      </c>
+      <c r="D23" s="5">
+        <f t="shared" si="1"/>
+        <v>37500000</v>
+      </c>
+      <c r="E23" s="4">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="F23" s="5"/>
+      <c r="G23" s="5"/>
+      <c r="H23" s="4">
+        <f t="shared" si="3"/>
+        <v>37500000</v>
+      </c>
+      <c r="I23" s="4">
+        <f t="shared" si="4"/>
+        <v>37500000</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+      <c r="A24" t="s">
+        <v>120</v>
+      </c>
+      <c r="B24" s="4"/>
+      <c r="C24" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="D24" s="5">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="E24" s="4" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F24" s="5"/>
+      <c r="G24" s="5"/>
+      <c r="H24" s="4" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="I24" s="4" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="25" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+      <c r="A25" t="s">
+        <v>121</v>
+      </c>
+      <c r="B25" s="4"/>
+      <c r="C25" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="D25" s="5">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="E25" s="4" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F25" s="5"/>
+      <c r="G25" s="5"/>
+      <c r="H25" s="4" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="I25" s="4" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A26" t="s">
+        <v>122</v>
+      </c>
+      <c r="B26" s="4">
+        <v>60000000</v>
+      </c>
+      <c r="C26" s="5">
+        <f t="shared" si="0"/>
+        <v>60000000</v>
+      </c>
+      <c r="D26" s="5">
+        <f t="shared" si="1"/>
+        <v>30000000</v>
+      </c>
+      <c r="E26" s="4">
+        <f t="shared" si="2"/>
+        <v>9000000</v>
+      </c>
+      <c r="F26" s="5"/>
+      <c r="G26" s="5">
+        <v>9000000</v>
+      </c>
+      <c r="H26" s="4">
+        <f t="shared" si="3"/>
+        <v>21000000</v>
+      </c>
+      <c r="I26" s="4">
+        <f t="shared" si="4"/>
+        <v>30000000</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A27" t="s">
+        <v>123</v>
+      </c>
+      <c r="B27" s="4">
+        <v>45150000</v>
+      </c>
+      <c r="C27" s="5">
+        <f t="shared" si="0"/>
+        <v>45150000</v>
+      </c>
+      <c r="D27" s="5">
+        <f t="shared" si="1"/>
+        <v>22575000</v>
+      </c>
+      <c r="E27" s="4">
+        <f t="shared" si="2"/>
+        <v>6423200</v>
+      </c>
+      <c r="F27" s="5">
+        <v>6119400</v>
+      </c>
+      <c r="G27" s="5">
+        <v>12542600</v>
+      </c>
+      <c r="H27" s="4">
+        <f t="shared" si="3"/>
+        <v>10032400</v>
+      </c>
+      <c r="I27" s="4">
+        <f t="shared" si="4"/>
+        <v>22575000</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+      <c r="A28" t="s">
+        <v>124</v>
+      </c>
+      <c r="B28" s="4"/>
+      <c r="C28" s="5"/>
+      <c r="D28" s="5"/>
+      <c r="E28" s="4" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F28" s="5"/>
+      <c r="G28" s="5"/>
+      <c r="H28" s="4" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="I28" s="4" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="29" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+      <c r="A29" t="s">
+        <v>125</v>
+      </c>
+      <c r="B29" s="4"/>
+      <c r="C29" s="5"/>
+      <c r="D29" s="5"/>
+      <c r="E29" s="4" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F29" s="5"/>
+      <c r="G29" s="5"/>
+      <c r="H29" s="4" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="I29" s="4" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="30" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+      <c r="A30" t="s">
+        <v>126</v>
+      </c>
+      <c r="B30" s="4"/>
+      <c r="C30" s="5"/>
+      <c r="D30" s="5"/>
+      <c r="E30" s="4" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F30" s="5"/>
+      <c r="G30" s="5"/>
+      <c r="H30" s="4" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="I30" s="4" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="31" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+      <c r="A31" t="s">
+        <v>127</v>
+      </c>
+      <c r="B31" s="4"/>
+      <c r="C31" s="5"/>
+      <c r="D31" s="5"/>
+      <c r="E31" s="4" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F31" s="5"/>
+      <c r="G31" s="5"/>
+      <c r="H31" s="4" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="I31" s="4" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="32" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+      <c r="A32" t="s">
+        <v>128</v>
+      </c>
+      <c r="B32" s="4"/>
+      <c r="C32" s="5"/>
+      <c r="D32" s="5"/>
+      <c r="E32" s="4" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F32" s="5"/>
+      <c r="G32" s="5"/>
+      <c r="H32" s="4" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="I32" s="4" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="33" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+      <c r="A33" t="s">
+        <v>129</v>
+      </c>
+      <c r="B33" s="4"/>
+      <c r="C33" s="5"/>
+      <c r="D33" s="5"/>
+      <c r="E33" s="4" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F33" s="5"/>
+      <c r="G33" s="5"/>
+      <c r="H33" s="4" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="I33" s="4" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A34" t="s">
+        <v>130</v>
+      </c>
+      <c r="B34" s="4">
+        <v>6000000</v>
+      </c>
+      <c r="C34" s="5">
+        <f>B34</f>
+        <v>6000000</v>
+      </c>
+      <c r="D34" s="5">
+        <f>C34/4</f>
+        <v>1500000</v>
+      </c>
+      <c r="E34" s="4">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="F34" s="5"/>
+      <c r="G34" s="5"/>
+      <c r="H34" s="4">
+        <f t="shared" si="3"/>
+        <v>1500000</v>
+      </c>
+      <c r="I34" s="4">
+        <f t="shared" si="4"/>
+        <v>4500000</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A35" t="s">
+        <v>131</v>
+      </c>
+      <c r="B35" s="4">
+        <v>41000000</v>
+      </c>
+      <c r="C35" s="5">
+        <f t="shared" ref="C35:C40" si="5">B35</f>
+        <v>41000000</v>
+      </c>
+      <c r="D35" s="5">
+        <f t="shared" ref="D35:D40" si="6">C35/4</f>
+        <v>10250000</v>
+      </c>
+      <c r="E35" s="4">
+        <f t="shared" si="2"/>
+        <v>1997700</v>
+      </c>
+      <c r="F35" s="5">
+        <v>998400</v>
+      </c>
+      <c r="G35" s="5">
+        <v>2996100</v>
+      </c>
+      <c r="H35" s="4">
+        <f t="shared" si="3"/>
+        <v>7253900</v>
+      </c>
+      <c r="I35" s="4">
+        <f t="shared" si="4"/>
+        <v>30750000</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A36" t="s">
+        <v>132</v>
+      </c>
+      <c r="B36" s="4">
+        <v>12000000</v>
+      </c>
+      <c r="C36" s="5">
+        <f t="shared" si="5"/>
+        <v>12000000</v>
+      </c>
+      <c r="D36" s="5">
+        <f t="shared" si="6"/>
+        <v>3000000</v>
+      </c>
+      <c r="E36" s="4">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="F36" s="5"/>
+      <c r="G36" s="5"/>
+      <c r="H36" s="4">
+        <f t="shared" si="3"/>
+        <v>3000000</v>
+      </c>
+      <c r="I36" s="4">
+        <f t="shared" si="4"/>
+        <v>9000000</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A37" t="s">
+        <v>133</v>
+      </c>
+      <c r="B37" s="4">
+        <v>171000000</v>
+      </c>
+      <c r="C37" s="5">
+        <f t="shared" si="5"/>
+        <v>171000000</v>
+      </c>
+      <c r="D37" s="5">
+        <f t="shared" si="6"/>
+        <v>42750000</v>
+      </c>
+      <c r="E37" s="4">
+        <f t="shared" si="2"/>
+        <v>5880000</v>
+      </c>
+      <c r="F37" s="5"/>
+      <c r="G37" s="5">
+        <v>5880000</v>
+      </c>
+      <c r="H37" s="4">
+        <f t="shared" si="3"/>
+        <v>36870000</v>
+      </c>
+      <c r="I37" s="4">
+        <f t="shared" si="4"/>
+        <v>128250000</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A38" t="s">
+        <v>134</v>
+      </c>
+      <c r="B38" s="4">
+        <v>130000000</v>
+      </c>
+      <c r="C38" s="5">
+        <f t="shared" si="5"/>
+        <v>130000000</v>
+      </c>
+      <c r="D38" s="5">
+        <f t="shared" si="6"/>
+        <v>32500000</v>
+      </c>
+      <c r="E38" s="4">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="F38" s="5">
+        <v>7381250</v>
+      </c>
+      <c r="G38" s="5">
+        <v>7381250</v>
+      </c>
+      <c r="H38" s="4">
+        <f t="shared" si="3"/>
+        <v>25118750</v>
+      </c>
+      <c r="I38" s="4">
+        <f t="shared" si="4"/>
+        <v>97500000</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A39" t="s">
+        <v>135</v>
+      </c>
+      <c r="B39" s="4">
+        <v>6660000</v>
+      </c>
+      <c r="C39" s="5">
+        <f t="shared" si="5"/>
+        <v>6660000</v>
+      </c>
+      <c r="D39" s="5">
+        <f t="shared" si="6"/>
+        <v>1665000</v>
+      </c>
+      <c r="E39" s="4">
+        <f t="shared" si="2"/>
+        <v>1665000</v>
+      </c>
+      <c r="F39" s="5"/>
+      <c r="G39" s="5">
+        <v>1665000</v>
+      </c>
+      <c r="H39" s="4">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="I39" s="4">
+        <f t="shared" si="4"/>
+        <v>4995000</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A40" t="s">
+        <v>136</v>
+      </c>
+      <c r="B40" s="4">
+        <v>6000000</v>
+      </c>
+      <c r="C40" s="5">
+        <f t="shared" si="5"/>
+        <v>6000000</v>
+      </c>
+      <c r="D40" s="5">
+        <f t="shared" si="6"/>
+        <v>1500000</v>
+      </c>
+      <c r="E40" s="4">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="F40" s="5"/>
+      <c r="G40" s="5"/>
+      <c r="H40" s="4">
+        <f t="shared" si="3"/>
+        <v>1500000</v>
+      </c>
+      <c r="I40" s="4">
+        <f t="shared" si="4"/>
+        <v>4500000</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+      <c r="A41" t="s">
+        <v>137</v>
+      </c>
+      <c r="B41" s="4"/>
+      <c r="C41" s="9"/>
+      <c r="D41" s="9"/>
+      <c r="E41" s="4" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F41" s="9"/>
+      <c r="G41" s="9"/>
+      <c r="H41" s="4" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="I41" s="4" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="42" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+      <c r="A42" t="s">
+        <v>138</v>
+      </c>
+      <c r="B42" s="4"/>
+      <c r="C42" s="9"/>
+      <c r="D42" s="9"/>
+      <c r="E42" s="4" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F42" s="9"/>
+      <c r="G42" s="9"/>
+      <c r="H42" s="4" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="I42" s="4" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="43" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+      <c r="A43" t="s">
+        <v>139</v>
+      </c>
+      <c r="B43" s="4"/>
+      <c r="C43" s="9"/>
+      <c r="D43" s="9"/>
+      <c r="E43" s="4" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F43" s="9"/>
+      <c r="G43" s="9"/>
+      <c r="H43" s="4" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="I43" s="4" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="44" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+      <c r="A44" t="s">
+        <v>140</v>
+      </c>
+      <c r="B44" s="4"/>
+      <c r="C44" s="9"/>
+      <c r="D44" s="9"/>
+      <c r="E44" s="4" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F44" s="9"/>
+      <c r="G44" s="9"/>
+      <c r="H44" s="4" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="I44" s="4" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="45" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+      <c r="A45" t="s">
+        <v>141</v>
+      </c>
+      <c r="B45" s="4"/>
+      <c r="C45" s="9"/>
+      <c r="D45" s="9"/>
+      <c r="E45" s="4" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F45" s="9"/>
+      <c r="G45" s="9"/>
+      <c r="H45" s="4" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="I45" s="4" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="46" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+      <c r="A46" t="s">
+        <v>142</v>
+      </c>
+      <c r="B46" s="4"/>
+      <c r="C46" s="9"/>
+      <c r="D46" s="9"/>
+      <c r="E46" s="4" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F46" s="9"/>
+      <c r="G46" s="9"/>
+      <c r="H46" s="4" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="I46" s="4" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="47" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+      <c r="A47" t="s">
+        <v>143</v>
+      </c>
+      <c r="B47" s="4"/>
+      <c r="C47" s="9"/>
+      <c r="D47" s="9"/>
+      <c r="E47" s="4" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F47" s="9"/>
+      <c r="G47" s="9"/>
+      <c r="H47" s="4" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="I47" s="4" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="48" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+      <c r="A48" t="s">
+        <v>144</v>
+      </c>
+      <c r="B48" s="4"/>
+      <c r="C48" s="9"/>
+      <c r="D48" s="9"/>
+      <c r="E48" s="4" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F48" s="9"/>
+      <c r="G48" s="9"/>
+      <c r="H48" s="4" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="I48" s="4" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="49" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+      <c r="A49" t="s">
+        <v>145</v>
+      </c>
+      <c r="B49" s="4"/>
+      <c r="C49" s="9"/>
+      <c r="D49" s="9"/>
+      <c r="E49" s="4" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F49" s="9"/>
+      <c r="G49" s="9"/>
+      <c r="H49" s="4" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="I49" s="4" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="50" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+      <c r="A50" t="s">
+        <v>146</v>
+      </c>
+      <c r="B50" s="4"/>
+      <c r="C50" s="9"/>
+      <c r="D50" s="9"/>
+      <c r="E50" s="4" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F50" s="9"/>
+      <c r="G50" s="9"/>
+      <c r="H50" s="4" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="I50" s="4" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="51" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+      <c r="A51" t="s">
+        <v>147</v>
+      </c>
+      <c r="B51" s="4"/>
+      <c r="C51" s="9"/>
+      <c r="D51" s="9"/>
+      <c r="E51" s="4" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F51" s="9"/>
+      <c r="G51" s="9"/>
+      <c r="H51" s="4" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="I51" s="4" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="52" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+      <c r="A52" t="s">
+        <v>148</v>
+      </c>
+      <c r="B52" s="4"/>
+      <c r="C52" s="9"/>
+      <c r="D52" s="9"/>
+      <c r="E52" s="4" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F52" s="9"/>
+      <c r="G52" s="9"/>
+      <c r="H52" s="4" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="I52" s="4" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="53" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+      <c r="A53" t="s">
+        <v>149</v>
+      </c>
+      <c r="B53" s="4"/>
+      <c r="C53" s="9"/>
+      <c r="D53" s="9"/>
+      <c r="E53" s="4" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F53" s="9"/>
+      <c r="G53" s="9"/>
+      <c r="H53" s="4" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="I53" s="4" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="54" spans="1:9" s="10" customFormat="1" x14ac:dyDescent="0.45">
+      <c r="A54" s="10" t="s">
+        <v>150</v>
+      </c>
+      <c r="B54" s="11">
+        <f>SUM(B2:B53)</f>
+        <v>2349761000</v>
+      </c>
+      <c r="C54" s="11">
+        <f t="shared" ref="C54:I54" si="7">SUM(C2:C53)</f>
+        <v>2349761000</v>
+      </c>
+      <c r="D54" s="11">
+        <f t="shared" si="7"/>
+        <v>1085685500</v>
+      </c>
+      <c r="E54" s="11">
+        <f t="shared" si="7"/>
+        <v>443295900</v>
+      </c>
+      <c r="F54" s="11">
+        <f t="shared" si="7"/>
+        <v>80000880</v>
+      </c>
+      <c r="G54" s="11">
+        <f t="shared" si="7"/>
+        <v>523296780</v>
+      </c>
+      <c r="H54" s="11">
+        <f t="shared" si="7"/>
+        <v>562388720</v>
+      </c>
+      <c r="I54" s="11">
+        <f t="shared" si="7"/>
+        <v>1264075500</v>
+      </c>
+    </row>
+  </sheetData>
+  <sheetProtection algorithmName="SHA-512" hashValue="1jAoxgEfH1v+py+BabjE1SWtZrOmBQzll5J+0nEkCC4zpdaAqkqUQlFy6oRCGkgRojK/rMDnTPHDGbW/CMwxXA==" saltValue="rHdoy6qRDxYzetfIY6x9cQ==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>